<commit_message>
Adjust approach movement template formatting
</commit_message>
<xml_diff>
--- a/templates/four_leg_tmc_report_template_approach_v2.xlsx
+++ b/templates/four_leg_tmc_report_template_approach_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyRD\tmc-processor-public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76E33117-32C5-4635-9C31-0B3453586197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80913C0-1336-4134-B837-CE0008521C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E96BB6DC-A3D4-4753-97D1-67BA99371C7D}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{E96BB6DC-A3D4-4753-97D1-67BA99371C7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -1018,9 +1018,6 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1148,6 +1145,27 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="24" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1155,6 +1173,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="7" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="5" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="19" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="15" fontId="12" fillId="2" borderId="23" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1204,41 +1237,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="26" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="2" borderId="19" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="24" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="12" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="3" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="7" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="6" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="10" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2941,8 +2941,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr bwMode="auto">
         <a:xfrm>
-          <a:off x="7630968" y="1953491"/>
-          <a:ext cx="697346" cy="886114"/>
+          <a:off x="7729105" y="1936173"/>
+          <a:ext cx="703118" cy="857250"/>
           <a:chOff x="7593874" y="108992292"/>
           <a:chExt cx="780088" cy="760870"/>
         </a:xfrm>
@@ -5760,50 +5760,50 @@
       <c r="AN1" s="6"/>
     </row>
     <row r="2" spans="2:40" ht="63.75" customHeight="1" thickBot="1">
-      <c r="B2" s="136" t="str">
+      <c r="B2" s="147" t="str">
         <f>"ข้อมูลปริมาณจราจรบริเวณทางแยก (Turning Movement Count)
 จุดนับรถที่ "</f>
         <v xml:space="preserve">ข้อมูลปริมาณจราจรบริเวณทางแยก (Turning Movement Count)
 จุดนับรถที่ </v>
       </c>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
-      <c r="E2" s="137"/>
-      <c r="F2" s="137"/>
-      <c r="G2" s="137"/>
-      <c r="H2" s="137"/>
-      <c r="I2" s="137"/>
-      <c r="J2" s="137"/>
-      <c r="K2" s="137"/>
-      <c r="L2" s="137"/>
-      <c r="M2" s="137"/>
-      <c r="N2" s="137"/>
-      <c r="O2" s="137"/>
-      <c r="P2" s="137"/>
-      <c r="Q2" s="137"/>
-      <c r="R2" s="137"/>
-      <c r="S2" s="137"/>
-      <c r="T2" s="137"/>
-      <c r="U2" s="137"/>
-      <c r="V2" s="137"/>
-      <c r="W2" s="137"/>
-      <c r="X2" s="137"/>
-      <c r="Y2" s="137"/>
-      <c r="Z2" s="137"/>
-      <c r="AA2" s="137"/>
-      <c r="AB2" s="137"/>
-      <c r="AC2" s="137"/>
-      <c r="AD2" s="137"/>
-      <c r="AE2" s="137"/>
-      <c r="AF2" s="137"/>
-      <c r="AG2" s="137"/>
-      <c r="AH2" s="137"/>
-      <c r="AI2" s="137"/>
-      <c r="AJ2" s="137"/>
-      <c r="AK2" s="137"/>
-      <c r="AL2" s="137"/>
-      <c r="AM2" s="137"/>
-      <c r="AN2" s="138"/>
+      <c r="C2" s="148"/>
+      <c r="D2" s="148"/>
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="148"/>
+      <c r="H2" s="148"/>
+      <c r="I2" s="148"/>
+      <c r="J2" s="148"/>
+      <c r="K2" s="148"/>
+      <c r="L2" s="148"/>
+      <c r="M2" s="148"/>
+      <c r="N2" s="148"/>
+      <c r="O2" s="148"/>
+      <c r="P2" s="148"/>
+      <c r="Q2" s="148"/>
+      <c r="R2" s="148"/>
+      <c r="S2" s="148"/>
+      <c r="T2" s="148"/>
+      <c r="U2" s="148"/>
+      <c r="V2" s="148"/>
+      <c r="W2" s="148"/>
+      <c r="X2" s="148"/>
+      <c r="Y2" s="148"/>
+      <c r="Z2" s="148"/>
+      <c r="AA2" s="148"/>
+      <c r="AB2" s="148"/>
+      <c r="AC2" s="148"/>
+      <c r="AD2" s="148"/>
+      <c r="AE2" s="148"/>
+      <c r="AF2" s="148"/>
+      <c r="AG2" s="148"/>
+      <c r="AH2" s="148"/>
+      <c r="AI2" s="148"/>
+      <c r="AJ2" s="148"/>
+      <c r="AK2" s="148"/>
+      <c r="AL2" s="148"/>
+      <c r="AM2" s="148"/>
+      <c r="AN2" s="149"/>
     </row>
     <row r="3" spans="2:40" s="7" customFormat="1" ht="15" customHeight="1">
       <c r="B3" s="8"/>
@@ -5848,25 +5848,25 @@
     </row>
     <row r="4" spans="2:40" s="7" customFormat="1" ht="15" customHeight="1">
       <c r="B4" s="12"/>
-      <c r="C4" s="139" t="s">
+      <c r="C4" s="150" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="139"/>
-      <c r="E4" s="140"/>
-      <c r="F4" s="140"/>
-      <c r="G4" s="140"/>
-      <c r="H4" s="140"/>
-      <c r="I4" s="140"/>
-      <c r="J4" s="140"/>
-      <c r="K4" s="140"/>
-      <c r="L4" s="140"/>
-      <c r="M4" s="140"/>
-      <c r="N4" s="140"/>
-      <c r="O4" s="140"/>
-      <c r="P4" s="140"/>
-      <c r="Q4" s="140"/>
-      <c r="R4" s="140"/>
-      <c r="S4" s="140"/>
+      <c r="D4" s="150"/>
+      <c r="E4" s="151"/>
+      <c r="F4" s="151"/>
+      <c r="G4" s="151"/>
+      <c r="H4" s="151"/>
+      <c r="I4" s="151"/>
+      <c r="J4" s="151"/>
+      <c r="K4" s="151"/>
+      <c r="L4" s="151"/>
+      <c r="M4" s="151"/>
+      <c r="N4" s="151"/>
+      <c r="O4" s="151"/>
+      <c r="P4" s="151"/>
+      <c r="Q4" s="151"/>
+      <c r="R4" s="151"/>
+      <c r="S4" s="151"/>
       <c r="T4" s="13"/>
       <c r="U4" s="13"/>
       <c r="V4" s="13"/>
@@ -5891,10 +5891,10 @@
     </row>
     <row r="5" spans="2:40" s="21" customFormat="1" ht="15" customHeight="1">
       <c r="B5" s="15"/>
-      <c r="C5" s="139" t="s">
+      <c r="C5" s="150" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="139"/>
+      <c r="D5" s="150"/>
       <c r="E5" s="16"/>
       <c r="F5" s="16"/>
       <c r="G5" s="16"/>
@@ -5903,16 +5903,16 @@
       <c r="J5" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="K5" s="141"/>
-      <c r="L5" s="142"/>
-      <c r="M5" s="142"/>
+      <c r="K5" s="152"/>
+      <c r="L5" s="153"/>
+      <c r="M5" s="153"/>
       <c r="N5" s="18"/>
-      <c r="O5" s="139" t="s">
+      <c r="O5" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="P5" s="139"/>
-      <c r="Q5" s="143"/>
-      <c r="R5" s="143"/>
+      <c r="P5" s="150"/>
+      <c r="Q5" s="154"/>
+      <c r="R5" s="154"/>
       <c r="S5" s="19"/>
       <c r="T5" s="18"/>
       <c r="U5" s="18"/>
@@ -5936,10 +5936,10 @@
     </row>
     <row r="6" spans="2:40" s="21" customFormat="1" ht="15" customHeight="1">
       <c r="B6" s="15"/>
-      <c r="C6" s="139" t="s">
+      <c r="C6" s="150" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="139"/>
+      <c r="D6" s="150"/>
       <c r="E6" s="24" t="s">
         <v>22</v>
       </c>
@@ -5950,9 +5950,9 @@
       <c r="J6" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="K6" s="143"/>
-      <c r="L6" s="143"/>
-      <c r="M6" s="143"/>
+      <c r="K6" s="154"/>
+      <c r="L6" s="154"/>
+      <c r="M6" s="154"/>
       <c r="N6" s="17"/>
       <c r="O6" s="20"/>
       <c r="P6" s="20"/>
@@ -6024,15 +6024,15 @@
     </row>
     <row r="8" spans="2:40" ht="15" customHeight="1" thickBot="1">
       <c r="B8" s="26"/>
-      <c r="C8" s="144">
+      <c r="C8" s="155">
         <f>E5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="145"/>
-      <c r="E8" s="145"/>
-      <c r="F8" s="145"/>
-      <c r="G8" s="145"/>
-      <c r="H8" s="146"/>
+      <c r="D8" s="156"/>
+      <c r="E8" s="156"/>
+      <c r="F8" s="156"/>
+      <c r="G8" s="156"/>
+      <c r="H8" s="157"/>
       <c r="I8" s="30"/>
       <c r="J8" s="30"/>
       <c r="K8" s="30"/>
@@ -6042,45 +6042,45 @@
       <c r="O8" s="31"/>
       <c r="P8" s="31"/>
       <c r="Q8" s="31"/>
-      <c r="R8" s="147"/>
-      <c r="S8" s="147"/>
+      <c r="R8" s="158"/>
+      <c r="S8" s="158"/>
       <c r="T8" s="32"/>
       <c r="U8" s="33"/>
-      <c r="V8" s="148" t="s">
+      <c r="V8" s="134" t="s">
         <v>24</v>
       </c>
-      <c r="W8" s="130" t="s">
+      <c r="W8" s="136" t="s">
         <v>25</v>
       </c>
-      <c r="X8" s="131"/>
-      <c r="Y8" s="131"/>
-      <c r="Z8" s="131"/>
-      <c r="AA8" s="131"/>
-      <c r="AB8" s="131"/>
-      <c r="AC8" s="131"/>
-      <c r="AD8" s="131"/>
-      <c r="AE8" s="131"/>
-      <c r="AF8" s="131"/>
-      <c r="AG8" s="131"/>
-      <c r="AH8" s="131"/>
-      <c r="AI8" s="131"/>
-      <c r="AJ8" s="131"/>
-      <c r="AK8" s="131"/>
-      <c r="AL8" s="131"/>
-      <c r="AM8" s="132"/>
+      <c r="X8" s="137"/>
+      <c r="Y8" s="137"/>
+      <c r="Z8" s="137"/>
+      <c r="AA8" s="137"/>
+      <c r="AB8" s="137"/>
+      <c r="AC8" s="137"/>
+      <c r="AD8" s="137"/>
+      <c r="AE8" s="137"/>
+      <c r="AF8" s="137"/>
+      <c r="AG8" s="137"/>
+      <c r="AH8" s="137"/>
+      <c r="AI8" s="137"/>
+      <c r="AJ8" s="137"/>
+      <c r="AK8" s="137"/>
+      <c r="AL8" s="137"/>
+      <c r="AM8" s="138"/>
       <c r="AN8" s="25"/>
     </row>
     <row r="9" spans="2:40" ht="15" customHeight="1" thickBot="1">
       <c r="B9" s="26"/>
-      <c r="C9" s="133">
+      <c r="C9" s="144">
         <f>+K5</f>
         <v>0</v>
       </c>
-      <c r="D9" s="134"/>
-      <c r="E9" s="134"/>
-      <c r="F9" s="134"/>
-      <c r="G9" s="134"/>
-      <c r="H9" s="135"/>
+      <c r="D9" s="145"/>
+      <c r="E9" s="145"/>
+      <c r="F9" s="145"/>
+      <c r="G9" s="145"/>
+      <c r="H9" s="146"/>
       <c r="I9" s="34"/>
       <c r="J9" s="34"/>
       <c r="K9" s="34"/>
@@ -6096,7 +6096,7 @@
       <c r="U9" s="37">
         <v>1</v>
       </c>
-      <c r="V9" s="149"/>
+      <c r="V9" s="135"/>
       <c r="W9" s="38" t="s">
         <v>55</v>
       </c>
@@ -6316,7 +6316,7 @@
       <c r="D12" s="28"/>
       <c r="E12" s="27"/>
       <c r="F12" s="27"/>
-      <c r="G12" s="34" t="s">
+      <c r="G12" s="10" t="s">
         <v>52</v>
       </c>
       <c r="H12" s="34"/>
@@ -6766,7 +6766,7 @@
       <c r="N17" s="27"/>
       <c r="O17" s="28"/>
       <c r="P17" s="28"/>
-      <c r="Q17" s="34" t="s">
+      <c r="Q17" s="10" t="s">
         <v>54</v>
       </c>
       <c r="R17" s="34"/>
@@ -7344,18 +7344,18 @@
       <c r="T23" s="54"/>
       <c r="U23" s="72"/>
       <c r="V23" s="72"/>
-      <c r="W23" s="150"/>
-      <c r="X23" s="150"/>
-      <c r="Y23" s="150"/>
-      <c r="Z23" s="150"/>
-      <c r="AA23" s="150"/>
-      <c r="AB23" s="150"/>
-      <c r="AC23" s="150"/>
-      <c r="AD23" s="150"/>
-      <c r="AE23" s="150"/>
-      <c r="AF23" s="150"/>
-      <c r="AG23" s="150"/>
-      <c r="AH23" s="150"/>
+      <c r="W23" s="142"/>
+      <c r="X23" s="142"/>
+      <c r="Y23" s="142"/>
+      <c r="Z23" s="142"/>
+      <c r="AA23" s="142"/>
+      <c r="AB23" s="142"/>
+      <c r="AC23" s="142"/>
+      <c r="AD23" s="142"/>
+      <c r="AE23" s="142"/>
+      <c r="AF23" s="142"/>
+      <c r="AG23" s="142"/>
+      <c r="AH23" s="142"/>
       <c r="AI23" s="72"/>
       <c r="AJ23" s="27"/>
       <c r="AK23" s="27"/>
@@ -7398,18 +7398,18 @@
       <c r="T24" s="62"/>
       <c r="U24" s="72"/>
       <c r="V24" s="27"/>
-      <c r="W24" s="151"/>
-      <c r="X24" s="151"/>
-      <c r="Y24" s="151"/>
-      <c r="Z24" s="151"/>
-      <c r="AA24" s="151"/>
-      <c r="AB24" s="151"/>
-      <c r="AC24" s="151"/>
-      <c r="AD24" s="151"/>
-      <c r="AE24" s="151"/>
-      <c r="AF24" s="151"/>
-      <c r="AG24" s="151"/>
-      <c r="AH24" s="151"/>
+      <c r="W24" s="143"/>
+      <c r="X24" s="143"/>
+      <c r="Y24" s="143"/>
+      <c r="Z24" s="143"/>
+      <c r="AA24" s="143"/>
+      <c r="AB24" s="143"/>
+      <c r="AC24" s="143"/>
+      <c r="AD24" s="143"/>
+      <c r="AE24" s="143"/>
+      <c r="AF24" s="143"/>
+      <c r="AG24" s="143"/>
+      <c r="AH24" s="143"/>
       <c r="AI24" s="27"/>
       <c r="AJ24" s="27"/>
       <c r="AK24" s="27"/>
@@ -7460,7 +7460,7 @@
     <row r="26" spans="2:40" ht="15" customHeight="1" thickBot="1">
       <c r="B26" s="42"/>
       <c r="C26" s="26"/>
-      <c r="D26" s="76" t="s">
+      <c r="D26" s="159" t="s">
         <v>51</v>
       </c>
       <c r="E26" s="34"/>
@@ -7477,28 +7477,28 @@
       <c r="P26" s="27"/>
       <c r="Q26" s="27"/>
       <c r="R26" s="27"/>
-      <c r="S26" s="77"/>
+      <c r="S26" s="76"/>
       <c r="T26" s="36"/>
       <c r="U26" s="33"/>
-      <c r="V26" s="148" t="s">
+      <c r="V26" s="134" t="s">
         <v>24</v>
       </c>
-      <c r="W26" s="130" t="s">
+      <c r="W26" s="136" t="s">
         <v>38</v>
       </c>
-      <c r="X26" s="131"/>
-      <c r="Y26" s="131"/>
-      <c r="Z26" s="131"/>
-      <c r="AA26" s="131"/>
-      <c r="AB26" s="131"/>
-      <c r="AC26" s="131"/>
-      <c r="AD26" s="131"/>
-      <c r="AE26" s="131"/>
-      <c r="AF26" s="131"/>
-      <c r="AG26" s="131"/>
-      <c r="AH26" s="131"/>
-      <c r="AI26" s="131"/>
-      <c r="AJ26" s="132"/>
+      <c r="X26" s="137"/>
+      <c r="Y26" s="137"/>
+      <c r="Z26" s="137"/>
+      <c r="AA26" s="137"/>
+      <c r="AB26" s="137"/>
+      <c r="AC26" s="137"/>
+      <c r="AD26" s="137"/>
+      <c r="AE26" s="137"/>
+      <c r="AF26" s="137"/>
+      <c r="AG26" s="137"/>
+      <c r="AH26" s="137"/>
+      <c r="AI26" s="137"/>
+      <c r="AJ26" s="138"/>
       <c r="AK26" s="27"/>
       <c r="AL26" s="27"/>
       <c r="AM26" s="27"/>
@@ -7506,7 +7506,7 @@
     </row>
     <row r="27" spans="2:40" ht="15" customHeight="1" thickBot="1">
       <c r="B27" s="42"/>
-      <c r="C27" s="78"/>
+      <c r="C27" s="77"/>
       <c r="E27" s="27"/>
       <c r="F27" s="27"/>
       <c r="G27" s="27"/>
@@ -7536,14 +7536,14 @@
       <c r="S27" s="35"/>
       <c r="T27" s="36"/>
       <c r="U27" s="33"/>
-      <c r="V27" s="149"/>
+      <c r="V27" s="135"/>
       <c r="W27" s="39" t="s">
         <v>39</v>
       </c>
       <c r="X27" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="Y27" s="79" t="s">
+      <c r="Y27" s="78" t="s">
         <v>14</v>
       </c>
       <c r="Z27" s="38" t="s">
@@ -7576,7 +7576,7 @@
       <c r="AI27" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="AJ27" s="80" t="s">
+      <c r="AJ27" s="79" t="s">
         <v>6</v>
       </c>
       <c r="AK27" s="27"/>
@@ -7616,7 +7616,7 @@
       <c r="R28" s="27"/>
       <c r="S28" s="35"/>
       <c r="T28" s="36"/>
-      <c r="U28" s="81"/>
+      <c r="U28" s="80"/>
       <c r="V28" s="45" t="s">
         <v>26</v>
       </c>
@@ -7625,18 +7625,18 @@
         <v>1171</v>
       </c>
       <c r="X28" s="46"/>
-      <c r="Y28" s="82"/>
-      <c r="Z28" s="83"/>
-      <c r="AA28" s="83"/>
-      <c r="AB28" s="83"/>
-      <c r="AC28" s="83"/>
-      <c r="AD28" s="83"/>
-      <c r="AE28" s="83"/>
-      <c r="AF28" s="84"/>
-      <c r="AG28" s="83"/>
-      <c r="AH28" s="83"/>
-      <c r="AI28" s="83"/>
-      <c r="AJ28" s="85"/>
+      <c r="Y28" s="81"/>
+      <c r="Z28" s="82"/>
+      <c r="AA28" s="82"/>
+      <c r="AB28" s="82"/>
+      <c r="AC28" s="82"/>
+      <c r="AD28" s="82"/>
+      <c r="AE28" s="82"/>
+      <c r="AF28" s="83"/>
+      <c r="AG28" s="82"/>
+      <c r="AH28" s="82"/>
+      <c r="AI28" s="82"/>
+      <c r="AJ28" s="84"/>
       <c r="AK28" s="27"/>
       <c r="AL28" s="27"/>
       <c r="AM28" s="27"/>
@@ -7683,18 +7683,18 @@
         <v>1238</v>
       </c>
       <c r="X29" s="46"/>
-      <c r="Y29" s="82"/>
-      <c r="Z29" s="83"/>
-      <c r="AA29" s="83"/>
-      <c r="AB29" s="83"/>
-      <c r="AC29" s="83"/>
-      <c r="AD29" s="83"/>
-      <c r="AE29" s="83"/>
-      <c r="AF29" s="84"/>
-      <c r="AG29" s="83"/>
-      <c r="AH29" s="83"/>
-      <c r="AI29" s="83"/>
-      <c r="AJ29" s="85"/>
+      <c r="Y29" s="81"/>
+      <c r="Z29" s="82"/>
+      <c r="AA29" s="82"/>
+      <c r="AB29" s="82"/>
+      <c r="AC29" s="82"/>
+      <c r="AD29" s="82"/>
+      <c r="AE29" s="82"/>
+      <c r="AF29" s="83"/>
+      <c r="AG29" s="82"/>
+      <c r="AH29" s="82"/>
+      <c r="AI29" s="82"/>
+      <c r="AJ29" s="84"/>
       <c r="AK29" s="27"/>
       <c r="AL29" s="27"/>
       <c r="AM29" s="27"/>
@@ -7703,15 +7703,15 @@
     <row r="30" spans="2:40" ht="15" customHeight="1">
       <c r="B30" s="26"/>
       <c r="C30" s="26"/>
-      <c r="D30" s="157" t="s">
+      <c r="D30" s="139" t="s">
         <v>41</v>
       </c>
-      <c r="E30" s="157"/>
-      <c r="F30" s="86">
+      <c r="E30" s="139"/>
+      <c r="F30" s="85">
         <f>SUM(G19:G22,J16:M16,O21:O24,J27:M27)</f>
         <v>1238</v>
       </c>
-      <c r="G30" s="87"/>
+      <c r="G30" s="86"/>
       <c r="H30" s="27"/>
       <c r="I30" s="27"/>
       <c r="J30" s="51" t="s">
@@ -7742,18 +7742,18 @@
         <v>1046</v>
       </c>
       <c r="X30" s="46"/>
-      <c r="Y30" s="82"/>
-      <c r="Z30" s="83"/>
-      <c r="AA30" s="83"/>
-      <c r="AB30" s="83"/>
-      <c r="AC30" s="83"/>
-      <c r="AD30" s="83"/>
-      <c r="AE30" s="83"/>
-      <c r="AF30" s="84"/>
-      <c r="AG30" s="83"/>
-      <c r="AH30" s="83"/>
-      <c r="AI30" s="83"/>
-      <c r="AJ30" s="85"/>
+      <c r="Y30" s="81"/>
+      <c r="Z30" s="82"/>
+      <c r="AA30" s="82"/>
+      <c r="AB30" s="82"/>
+      <c r="AC30" s="82"/>
+      <c r="AD30" s="82"/>
+      <c r="AE30" s="82"/>
+      <c r="AF30" s="83"/>
+      <c r="AG30" s="82"/>
+      <c r="AH30" s="82"/>
+      <c r="AI30" s="82"/>
+      <c r="AJ30" s="84"/>
       <c r="AK30" s="27"/>
       <c r="AL30" s="27"/>
       <c r="AM30" s="27"/>
@@ -7762,15 +7762,15 @@
     <row r="31" spans="2:40" ht="15" customHeight="1">
       <c r="B31" s="42"/>
       <c r="C31" s="26"/>
-      <c r="D31" s="158" t="s">
+      <c r="D31" s="140" t="s">
         <v>42</v>
       </c>
-      <c r="E31" s="158"/>
+      <c r="E31" s="140"/>
       <c r="F31" s="55">
         <f>SUM(J15:M15,F19:F22,J28:M28,P21:P24)</f>
         <v>1312</v>
       </c>
-      <c r="G31" s="87"/>
+      <c r="G31" s="86"/>
       <c r="H31" s="27"/>
       <c r="I31" s="27"/>
       <c r="J31" s="27"/>
@@ -7784,7 +7784,7 @@
       <c r="R31" s="27"/>
       <c r="S31" s="27"/>
       <c r="T31" s="36"/>
-      <c r="U31" s="81"/>
+      <c r="U31" s="80"/>
       <c r="V31" s="45" t="s">
         <v>29</v>
       </c>
@@ -7793,18 +7793,18 @@
         <v>1097</v>
       </c>
       <c r="X31" s="46"/>
-      <c r="Y31" s="82"/>
-      <c r="Z31" s="83"/>
-      <c r="AA31" s="83"/>
-      <c r="AB31" s="83"/>
-      <c r="AC31" s="83"/>
-      <c r="AD31" s="83"/>
-      <c r="AE31" s="83"/>
-      <c r="AF31" s="84"/>
-      <c r="AG31" s="83"/>
-      <c r="AH31" s="83"/>
-      <c r="AI31" s="83"/>
-      <c r="AJ31" s="85"/>
+      <c r="Y31" s="81"/>
+      <c r="Z31" s="82"/>
+      <c r="AA31" s="82"/>
+      <c r="AB31" s="82"/>
+      <c r="AC31" s="82"/>
+      <c r="AD31" s="82"/>
+      <c r="AE31" s="82"/>
+      <c r="AF31" s="83"/>
+      <c r="AG31" s="82"/>
+      <c r="AH31" s="82"/>
+      <c r="AI31" s="82"/>
+      <c r="AJ31" s="84"/>
       <c r="AK31" s="27"/>
       <c r="AL31" s="27"/>
       <c r="AM31" s="27"/>
@@ -7813,10 +7813,10 @@
     <row r="32" spans="2:40" ht="15" customHeight="1">
       <c r="B32" s="42"/>
       <c r="C32" s="26"/>
-      <c r="D32" s="159" t="s">
+      <c r="D32" s="141" t="s">
         <v>43</v>
       </c>
-      <c r="E32" s="159"/>
+      <c r="E32" s="141"/>
       <c r="F32" s="53">
         <f>SUM(J14:M14,E19:E22,J29:M29,Q21:Q24)</f>
         <v>14038</v>
@@ -7830,7 +7830,7 @@
       </c>
       <c r="L32" s="27"/>
       <c r="M32" s="27"/>
-      <c r="N32" s="129"/>
+      <c r="N32" s="128"/>
       <c r="O32" s="27" t="s">
         <v>53</v>
       </c>
@@ -7840,7 +7840,7 @@
       <c r="S32" s="27"/>
       <c r="T32" s="36"/>
       <c r="U32" s="33"/>
-      <c r="V32" s="88" t="s">
+      <c r="V32" s="87" t="s">
         <v>30</v>
       </c>
       <c r="W32" s="46">
@@ -7848,18 +7848,18 @@
         <v>1146</v>
       </c>
       <c r="X32" s="46"/>
-      <c r="Y32" s="89"/>
-      <c r="Z32" s="90"/>
-      <c r="AA32" s="90"/>
-      <c r="AB32" s="90"/>
-      <c r="AC32" s="90"/>
-      <c r="AD32" s="90"/>
-      <c r="AE32" s="90"/>
-      <c r="AF32" s="91"/>
-      <c r="AG32" s="90"/>
-      <c r="AH32" s="90"/>
-      <c r="AI32" s="90"/>
-      <c r="AJ32" s="92"/>
+      <c r="Y32" s="88"/>
+      <c r="Z32" s="89"/>
+      <c r="AA32" s="89"/>
+      <c r="AB32" s="89"/>
+      <c r="AC32" s="89"/>
+      <c r="AD32" s="89"/>
+      <c r="AE32" s="89"/>
+      <c r="AF32" s="90"/>
+      <c r="AG32" s="89"/>
+      <c r="AH32" s="89"/>
+      <c r="AI32" s="89"/>
+      <c r="AJ32" s="91"/>
       <c r="AK32" s="27"/>
       <c r="AL32" s="27"/>
       <c r="AM32" s="27"/>
@@ -7868,10 +7868,10 @@
     <row r="33" spans="2:53" ht="15" customHeight="1">
       <c r="B33" s="26"/>
       <c r="C33" s="42"/>
-      <c r="D33" s="152" t="s">
+      <c r="D33" s="129" t="s">
         <v>44</v>
       </c>
-      <c r="E33" s="152"/>
+      <c r="E33" s="129"/>
       <c r="F33" s="27"/>
       <c r="G33" s="27"/>
       <c r="H33" s="27"/>
@@ -7886,8 +7886,8 @@
       <c r="Q33" s="27"/>
       <c r="R33" s="27"/>
       <c r="S33" s="27"/>
-      <c r="T33" s="93"/>
-      <c r="U33" s="94"/>
+      <c r="T33" s="92"/>
+      <c r="U33" s="93"/>
       <c r="V33" s="45" t="s">
         <v>31</v>
       </c>
@@ -7896,18 +7896,18 @@
         <v>1218</v>
       </c>
       <c r="X33" s="46"/>
-      <c r="Y33" s="82"/>
-      <c r="Z33" s="83"/>
-      <c r="AA33" s="83"/>
-      <c r="AB33" s="83"/>
-      <c r="AC33" s="83"/>
-      <c r="AD33" s="83"/>
-      <c r="AE33" s="83"/>
-      <c r="AF33" s="84"/>
-      <c r="AG33" s="83"/>
-      <c r="AH33" s="83"/>
-      <c r="AI33" s="83"/>
-      <c r="AJ33" s="85"/>
+      <c r="Y33" s="81"/>
+      <c r="Z33" s="82"/>
+      <c r="AA33" s="82"/>
+      <c r="AB33" s="82"/>
+      <c r="AC33" s="82"/>
+      <c r="AD33" s="82"/>
+      <c r="AE33" s="82"/>
+      <c r="AF33" s="83"/>
+      <c r="AG33" s="82"/>
+      <c r="AH33" s="82"/>
+      <c r="AI33" s="82"/>
+      <c r="AJ33" s="84"/>
       <c r="AK33" s="27"/>
       <c r="AL33" s="27"/>
       <c r="AM33" s="27"/>
@@ -7917,23 +7917,23 @@
       <c r="B34" s="26"/>
       <c r="C34" s="26"/>
       <c r="D34" s="27"/>
-      <c r="E34" s="77"/>
-      <c r="F34" s="77"/>
-      <c r="G34" s="77"/>
-      <c r="H34" s="77"/>
-      <c r="I34" s="77"/>
-      <c r="J34" s="77"/>
-      <c r="K34" s="77"/>
-      <c r="L34" s="77"/>
-      <c r="M34" s="77"/>
-      <c r="N34" s="77"/>
-      <c r="O34" s="77"/>
-      <c r="P34" s="77"/>
-      <c r="Q34" s="77"/>
-      <c r="R34" s="77"/>
-      <c r="S34" s="95"/>
-      <c r="T34" s="93"/>
-      <c r="U34" s="94"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="76"/>
+      <c r="I34" s="76"/>
+      <c r="J34" s="76"/>
+      <c r="K34" s="76"/>
+      <c r="L34" s="76"/>
+      <c r="M34" s="76"/>
+      <c r="N34" s="76"/>
+      <c r="O34" s="76"/>
+      <c r="P34" s="76"/>
+      <c r="Q34" s="76"/>
+      <c r="R34" s="76"/>
+      <c r="S34" s="94"/>
+      <c r="T34" s="92"/>
+      <c r="U34" s="93"/>
       <c r="V34" s="45" t="s">
         <v>32</v>
       </c>
@@ -7942,18 +7942,18 @@
         <v>1099</v>
       </c>
       <c r="X34" s="46"/>
-      <c r="Y34" s="82"/>
-      <c r="Z34" s="83"/>
-      <c r="AA34" s="83"/>
-      <c r="AB34" s="83"/>
-      <c r="AC34" s="83"/>
-      <c r="AD34" s="83"/>
-      <c r="AE34" s="83"/>
-      <c r="AF34" s="84"/>
-      <c r="AG34" s="83"/>
-      <c r="AH34" s="83"/>
-      <c r="AI34" s="83"/>
-      <c r="AJ34" s="85"/>
+      <c r="Y34" s="81"/>
+      <c r="Z34" s="82"/>
+      <c r="AA34" s="82"/>
+      <c r="AB34" s="82"/>
+      <c r="AC34" s="82"/>
+      <c r="AD34" s="82"/>
+      <c r="AE34" s="82"/>
+      <c r="AF34" s="83"/>
+      <c r="AG34" s="82"/>
+      <c r="AH34" s="82"/>
+      <c r="AI34" s="82"/>
+      <c r="AJ34" s="84"/>
       <c r="AK34" s="27"/>
       <c r="AL34" s="27"/>
       <c r="AM34" s="27"/>
@@ -7963,22 +7963,22 @@
       <c r="B35" s="26"/>
       <c r="C35" s="26"/>
       <c r="D35" s="27"/>
-      <c r="E35" s="153" t="s">
+      <c r="E35" s="130" t="s">
         <v>45</v>
       </c>
-      <c r="F35" s="153"/>
-      <c r="G35" s="153"/>
-      <c r="H35" s="153"/>
-      <c r="I35" s="153"/>
-      <c r="J35" s="153"/>
-      <c r="K35" s="153"/>
-      <c r="L35" s="153"/>
-      <c r="M35" s="153"/>
-      <c r="N35" s="153"/>
-      <c r="O35" s="153"/>
-      <c r="P35" s="153"/>
-      <c r="Q35" s="153"/>
-      <c r="R35" s="153"/>
+      <c r="F35" s="130"/>
+      <c r="G35" s="130"/>
+      <c r="H35" s="130"/>
+      <c r="I35" s="130"/>
+      <c r="J35" s="130"/>
+      <c r="K35" s="130"/>
+      <c r="L35" s="130"/>
+      <c r="M35" s="130"/>
+      <c r="N35" s="130"/>
+      <c r="O35" s="130"/>
+      <c r="P35" s="130"/>
+      <c r="Q35" s="130"/>
+      <c r="R35" s="130"/>
       <c r="S35" s="27"/>
       <c r="T35" s="58"/>
       <c r="U35" s="27"/>
@@ -7990,18 +7990,18 @@
         <v>1146</v>
       </c>
       <c r="X35" s="46"/>
-      <c r="Y35" s="82"/>
-      <c r="Z35" s="83"/>
-      <c r="AA35" s="83"/>
-      <c r="AB35" s="83"/>
-      <c r="AC35" s="83"/>
-      <c r="AD35" s="83"/>
-      <c r="AE35" s="83"/>
-      <c r="AF35" s="84"/>
-      <c r="AG35" s="83"/>
-      <c r="AH35" s="83"/>
-      <c r="AI35" s="83"/>
-      <c r="AJ35" s="85"/>
+      <c r="Y35" s="81"/>
+      <c r="Z35" s="82"/>
+      <c r="AA35" s="82"/>
+      <c r="AB35" s="82"/>
+      <c r="AC35" s="82"/>
+      <c r="AD35" s="82"/>
+      <c r="AE35" s="82"/>
+      <c r="AF35" s="83"/>
+      <c r="AG35" s="82"/>
+      <c r="AH35" s="82"/>
+      <c r="AI35" s="82"/>
+      <c r="AJ35" s="84"/>
       <c r="AK35" s="27"/>
       <c r="AL35" s="27"/>
       <c r="AM35" s="27"/>
@@ -8009,26 +8009,26 @@
     </row>
     <row r="36" spans="2:53" ht="15" customHeight="1" thickBot="1">
       <c r="B36" s="42"/>
-      <c r="C36" s="98"/>
-      <c r="D36" s="99"/>
-      <c r="E36" s="154"/>
-      <c r="F36" s="154"/>
-      <c r="G36" s="154"/>
-      <c r="H36" s="154"/>
-      <c r="I36" s="154"/>
-      <c r="J36" s="154"/>
-      <c r="K36" s="154"/>
-      <c r="L36" s="154"/>
-      <c r="M36" s="154"/>
-      <c r="N36" s="154"/>
-      <c r="O36" s="154"/>
-      <c r="P36" s="154"/>
-      <c r="Q36" s="154"/>
-      <c r="R36" s="154"/>
-      <c r="S36" s="100"/>
-      <c r="T36" s="101"/>
+      <c r="C36" s="97"/>
+      <c r="D36" s="98"/>
+      <c r="E36" s="131"/>
+      <c r="F36" s="131"/>
+      <c r="G36" s="131"/>
+      <c r="H36" s="131"/>
+      <c r="I36" s="131"/>
+      <c r="J36" s="131"/>
+      <c r="K36" s="131"/>
+      <c r="L36" s="131"/>
+      <c r="M36" s="131"/>
+      <c r="N36" s="131"/>
+      <c r="O36" s="131"/>
+      <c r="P36" s="131"/>
+      <c r="Q36" s="131"/>
+      <c r="R36" s="131"/>
+      <c r="S36" s="99"/>
+      <c r="T36" s="100"/>
       <c r="U36" s="33"/>
-      <c r="V36" s="88" t="s">
+      <c r="V36" s="87" t="s">
         <v>34</v>
       </c>
       <c r="W36" s="46">
@@ -8036,18 +8036,18 @@
         <v>1256</v>
       </c>
       <c r="X36" s="46"/>
-      <c r="Y36" s="89"/>
-      <c r="Z36" s="90"/>
-      <c r="AA36" s="90"/>
-      <c r="AB36" s="90"/>
-      <c r="AC36" s="90"/>
-      <c r="AD36" s="90"/>
-      <c r="AE36" s="90"/>
-      <c r="AF36" s="91"/>
-      <c r="AG36" s="90"/>
-      <c r="AH36" s="90"/>
-      <c r="AI36" s="90"/>
-      <c r="AJ36" s="92"/>
+      <c r="Y36" s="88"/>
+      <c r="Z36" s="89"/>
+      <c r="AA36" s="89"/>
+      <c r="AB36" s="89"/>
+      <c r="AC36" s="89"/>
+      <c r="AD36" s="89"/>
+      <c r="AE36" s="89"/>
+      <c r="AF36" s="90"/>
+      <c r="AG36" s="89"/>
+      <c r="AH36" s="89"/>
+      <c r="AI36" s="89"/>
+      <c r="AJ36" s="91"/>
       <c r="AK36" s="27"/>
       <c r="AL36" s="27"/>
       <c r="AM36" s="27"/>
@@ -8082,18 +8082,18 @@
         <v>1243</v>
       </c>
       <c r="X37" s="46"/>
-      <c r="Y37" s="82"/>
-      <c r="Z37" s="83"/>
-      <c r="AA37" s="83"/>
-      <c r="AB37" s="83"/>
-      <c r="AC37" s="83"/>
-      <c r="AD37" s="83"/>
-      <c r="AE37" s="83"/>
-      <c r="AF37" s="84"/>
-      <c r="AG37" s="83"/>
-      <c r="AH37" s="83"/>
-      <c r="AI37" s="83"/>
-      <c r="AJ37" s="85"/>
+      <c r="Y37" s="81"/>
+      <c r="Z37" s="82"/>
+      <c r="AA37" s="82"/>
+      <c r="AB37" s="82"/>
+      <c r="AC37" s="82"/>
+      <c r="AD37" s="82"/>
+      <c r="AE37" s="82"/>
+      <c r="AF37" s="83"/>
+      <c r="AG37" s="82"/>
+      <c r="AH37" s="82"/>
+      <c r="AI37" s="82"/>
+      <c r="AJ37" s="84"/>
       <c r="AK37" s="27"/>
       <c r="AL37" s="27"/>
       <c r="AM37" s="27"/>
@@ -8128,67 +8128,67 @@
         <v>1311</v>
       </c>
       <c r="X38" s="46"/>
-      <c r="Y38" s="82"/>
-      <c r="Z38" s="83"/>
-      <c r="AA38" s="83"/>
-      <c r="AB38" s="83"/>
-      <c r="AC38" s="83"/>
-      <c r="AD38" s="83"/>
-      <c r="AE38" s="83"/>
-      <c r="AF38" s="84"/>
-      <c r="AG38" s="83"/>
-      <c r="AH38" s="83"/>
-      <c r="AI38" s="83"/>
-      <c r="AJ38" s="85"/>
+      <c r="Y38" s="81"/>
+      <c r="Z38" s="82"/>
+      <c r="AA38" s="82"/>
+      <c r="AB38" s="82"/>
+      <c r="AC38" s="82"/>
+      <c r="AD38" s="82"/>
+      <c r="AE38" s="82"/>
+      <c r="AF38" s="83"/>
+      <c r="AG38" s="82"/>
+      <c r="AH38" s="82"/>
+      <c r="AI38" s="82"/>
+      <c r="AJ38" s="84"/>
       <c r="AK38" s="27"/>
       <c r="AL38" s="27"/>
       <c r="AM38" s="27"/>
       <c r="AN38" s="58"/>
-      <c r="AP38" s="127">
+      <c r="AP38" s="126">
         <f t="shared" ref="AP38:BA38" si="7">Y40</f>
         <v>0</v>
       </c>
-      <c r="AQ38" s="127">
+      <c r="AQ38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AR38" s="127">
+      <c r="AR38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AS38" s="127">
+      <c r="AS38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AT38" s="127">
+      <c r="AT38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AU38" s="127">
+      <c r="AU38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AV38" s="127">
+      <c r="AV38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AW38" s="127">
+      <c r="AW38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AX38" s="127">
+      <c r="AX38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AY38" s="127">
+      <c r="AY38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="AZ38" s="127">
+      <c r="AZ38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="BA38" s="127">
+      <c r="BA38" s="126">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -8214,7 +8214,7 @@
       <c r="S39" s="27"/>
       <c r="T39" s="27"/>
       <c r="U39" s="27"/>
-      <c r="V39" s="88" t="s">
+      <c r="V39" s="87" t="s">
         <v>37</v>
       </c>
       <c r="W39" s="46">
@@ -8222,18 +8222,18 @@
         <v>1062</v>
       </c>
       <c r="X39" s="46"/>
-      <c r="Y39" s="89"/>
-      <c r="Z39" s="90"/>
-      <c r="AA39" s="90"/>
-      <c r="AB39" s="90"/>
-      <c r="AC39" s="90"/>
-      <c r="AD39" s="90"/>
-      <c r="AE39" s="90"/>
-      <c r="AF39" s="91"/>
-      <c r="AG39" s="90"/>
-      <c r="AH39" s="90"/>
-      <c r="AI39" s="90"/>
-      <c r="AJ39" s="92"/>
+      <c r="Y39" s="88"/>
+      <c r="Z39" s="89"/>
+      <c r="AA39" s="89"/>
+      <c r="AB39" s="89"/>
+      <c r="AC39" s="89"/>
+      <c r="AD39" s="89"/>
+      <c r="AE39" s="89"/>
+      <c r="AF39" s="90"/>
+      <c r="AG39" s="89"/>
+      <c r="AH39" s="89"/>
+      <c r="AI39" s="89"/>
+      <c r="AJ39" s="91"/>
       <c r="AK39" s="27"/>
       <c r="AL39" s="27"/>
       <c r="AM39" s="27"/>
@@ -8296,7 +8296,7 @@
       <c r="S40" s="27"/>
       <c r="T40" s="27"/>
       <c r="U40" s="27"/>
-      <c r="V40" s="102" t="s">
+      <c r="V40" s="101" t="s">
         <v>0</v>
       </c>
       <c r="W40" s="68">
@@ -8307,7 +8307,7 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="Y40" s="103">
+      <c r="Y40" s="102">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -8339,15 +8339,15 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AG40" s="104">
+      <c r="AG40" s="103">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AH40" s="104">
+      <c r="AH40" s="103">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="AI40" s="104">
+      <c r="AI40" s="103">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
@@ -8359,51 +8359,51 @@
       <c r="AL40" s="27"/>
       <c r="AM40" s="27"/>
       <c r="AN40" s="58"/>
-      <c r="AP40" s="128">
+      <c r="AP40" s="127">
         <f>IFERROR(AP38/SUM($AP$38:$BA$38),0)</f>
         <v>0</v>
       </c>
-      <c r="AQ40" s="128">
+      <c r="AQ40" s="127">
         <f t="shared" ref="AQ40:BA40" si="9">IFERROR(AQ38/SUM($AP$38:$BA$38),0)</f>
         <v>0</v>
       </c>
-      <c r="AR40" s="128">
+      <c r="AR40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AS40" s="128">
+      <c r="AS40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AT40" s="128">
+      <c r="AT40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AU40" s="128">
+      <c r="AU40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AV40" s="128">
+      <c r="AV40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AW40" s="128">
+      <c r="AW40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AX40" s="128">
+      <c r="AX40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AY40" s="128">
+      <c r="AY40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AZ40" s="128">
+      <c r="AZ40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="BA40" s="128">
+      <c r="BA40" s="127">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -8430,16 +8430,16 @@
       <c r="T41" s="27"/>
       <c r="U41" s="27"/>
       <c r="V41" s="27"/>
-      <c r="W41" s="105"/>
-      <c r="X41" s="106"/>
-      <c r="Y41" s="107"/>
-      <c r="Z41" s="108"/>
-      <c r="AA41" s="108"/>
-      <c r="AB41" s="108"/>
-      <c r="AC41" s="108"/>
-      <c r="AD41" s="108"/>
-      <c r="AE41" s="108"/>
-      <c r="AF41" s="108"/>
+      <c r="W41" s="104"/>
+      <c r="X41" s="105"/>
+      <c r="Y41" s="106"/>
+      <c r="Z41" s="107"/>
+      <c r="AA41" s="107"/>
+      <c r="AB41" s="107"/>
+      <c r="AC41" s="107"/>
+      <c r="AD41" s="107"/>
+      <c r="AE41" s="107"/>
+      <c r="AF41" s="107"/>
       <c r="AG41" s="27"/>
       <c r="AH41" s="27"/>
       <c r="AI41" s="27"/>
@@ -8594,16 +8594,16 @@
       <c r="T45" s="27"/>
       <c r="U45" s="27"/>
       <c r="V45" s="27"/>
-      <c r="W45" s="105"/>
-      <c r="X45" s="106"/>
-      <c r="Y45" s="107"/>
-      <c r="Z45" s="108"/>
-      <c r="AA45" s="108"/>
-      <c r="AB45" s="108"/>
-      <c r="AC45" s="108"/>
-      <c r="AD45" s="108"/>
-      <c r="AE45" s="108"/>
-      <c r="AF45" s="108"/>
+      <c r="W45" s="104"/>
+      <c r="X45" s="105"/>
+      <c r="Y45" s="106"/>
+      <c r="Z45" s="107"/>
+      <c r="AA45" s="107"/>
+      <c r="AB45" s="107"/>
+      <c r="AC45" s="107"/>
+      <c r="AD45" s="107"/>
+      <c r="AE45" s="107"/>
+      <c r="AF45" s="107"/>
       <c r="AG45" s="27"/>
       <c r="AH45" s="27"/>
       <c r="AI45" s="27"/>
@@ -8932,9 +8932,9 @@
       <c r="AD53" s="27"/>
       <c r="AE53" s="27"/>
       <c r="AF53" s="27"/>
-      <c r="AG53" s="109"/>
-      <c r="AH53" s="109"/>
-      <c r="AI53" s="109"/>
+      <c r="AG53" s="108"/>
+      <c r="AH53" s="108"/>
+      <c r="AI53" s="108"/>
       <c r="AJ53" s="27"/>
       <c r="AK53" s="27"/>
       <c r="AL53" s="27"/>
@@ -8973,10 +8973,10 @@
       <c r="AD54" s="27"/>
       <c r="AE54" s="27"/>
       <c r="AF54" s="27"/>
-      <c r="AG54" s="109"/>
-      <c r="AH54" s="109"/>
-      <c r="AI54" s="109"/>
-      <c r="AJ54" s="110"/>
+      <c r="AG54" s="108"/>
+      <c r="AH54" s="108"/>
+      <c r="AI54" s="108"/>
+      <c r="AJ54" s="109"/>
       <c r="AK54" s="27"/>
       <c r="AL54" s="27"/>
       <c r="AM54" s="27"/>
@@ -9014,7 +9014,7 @@
       <c r="AD55" s="27"/>
       <c r="AE55" s="27"/>
       <c r="AF55" s="27"/>
-      <c r="AG55" s="109"/>
+      <c r="AG55" s="108"/>
       <c r="AH55" s="27"/>
       <c r="AI55" s="27"/>
       <c r="AJ55" s="27"/>
@@ -9126,17 +9126,17 @@
       <c r="S58" s="27"/>
       <c r="T58" s="27"/>
       <c r="U58" s="27"/>
-      <c r="V58" s="94"/>
-      <c r="W58" s="109"/>
-      <c r="X58" s="109"/>
-      <c r="Y58" s="109"/>
-      <c r="Z58" s="109"/>
-      <c r="AA58" s="109"/>
-      <c r="AB58" s="109"/>
-      <c r="AC58" s="109"/>
-      <c r="AD58" s="109"/>
-      <c r="AE58" s="109"/>
-      <c r="AF58" s="109"/>
+      <c r="V58" s="93"/>
+      <c r="W58" s="108"/>
+      <c r="X58" s="108"/>
+      <c r="Y58" s="108"/>
+      <c r="Z58" s="108"/>
+      <c r="AA58" s="108"/>
+      <c r="AB58" s="108"/>
+      <c r="AC58" s="108"/>
+      <c r="AD58" s="108"/>
+      <c r="AE58" s="108"/>
+      <c r="AF58" s="108"/>
       <c r="AG58" s="27"/>
       <c r="AH58" s="27"/>
       <c r="AI58" s="27"/>
@@ -9178,8 +9178,8 @@
       <c r="AD59" s="27"/>
       <c r="AE59" s="27"/>
       <c r="AF59" s="27"/>
-      <c r="AG59" s="111"/>
-      <c r="AH59" s="111"/>
+      <c r="AG59" s="110"/>
+      <c r="AH59" s="110"/>
       <c r="AI59" s="27"/>
       <c r="AJ59" s="27"/>
       <c r="AK59" s="27"/>
@@ -9229,40 +9229,40 @@
       <c r="AN60" s="58"/>
     </row>
     <row r="61" spans="2:40" ht="15" customHeight="1">
-      <c r="B61" s="155" t="s">
+      <c r="B61" s="132" t="s">
         <v>46</v>
       </c>
-      <c r="C61" s="156"/>
-      <c r="D61" s="156"/>
-      <c r="E61" s="156"/>
-      <c r="F61" s="156"/>
-      <c r="G61" s="156"/>
-      <c r="H61" s="156"/>
-      <c r="I61" s="156"/>
-      <c r="J61" s="156"/>
-      <c r="K61" s="156"/>
-      <c r="L61" s="156"/>
-      <c r="M61" s="156"/>
-      <c r="N61" s="156"/>
-      <c r="O61" s="156"/>
-      <c r="P61" s="156"/>
-      <c r="Q61" s="156"/>
-      <c r="R61" s="156"/>
-      <c r="S61" s="156"/>
-      <c r="T61" s="156"/>
-      <c r="U61" s="156"/>
+      <c r="C61" s="133"/>
+      <c r="D61" s="133"/>
+      <c r="E61" s="133"/>
+      <c r="F61" s="133"/>
+      <c r="G61" s="133"/>
+      <c r="H61" s="133"/>
+      <c r="I61" s="133"/>
+      <c r="J61" s="133"/>
+      <c r="K61" s="133"/>
+      <c r="L61" s="133"/>
+      <c r="M61" s="133"/>
+      <c r="N61" s="133"/>
+      <c r="O61" s="133"/>
+      <c r="P61" s="133"/>
+      <c r="Q61" s="133"/>
+      <c r="R61" s="133"/>
+      <c r="S61" s="133"/>
+      <c r="T61" s="133"/>
+      <c r="U61" s="133"/>
       <c r="V61" s="27"/>
-      <c r="W61" s="112"/>
-      <c r="X61" s="97"/>
-      <c r="Y61" s="97"/>
-      <c r="Z61" s="112"/>
-      <c r="AA61" s="112"/>
+      <c r="W61" s="111"/>
+      <c r="X61" s="96"/>
+      <c r="Y61" s="96"/>
+      <c r="Z61" s="111"/>
+      <c r="AA61" s="111"/>
       <c r="AB61" s="27"/>
-      <c r="AC61" s="111"/>
-      <c r="AD61" s="111"/>
-      <c r="AE61" s="111"/>
-      <c r="AF61" s="110"/>
-      <c r="AG61" s="110"/>
+      <c r="AC61" s="110"/>
+      <c r="AD61" s="110"/>
+      <c r="AE61" s="110"/>
+      <c r="AF61" s="109"/>
+      <c r="AG61" s="109"/>
       <c r="AH61" s="27"/>
       <c r="AI61" s="27"/>
       <c r="AJ61" s="27"/>
@@ -9272,37 +9272,37 @@
       <c r="AN61" s="58"/>
     </row>
     <row r="62" spans="2:40" ht="15" customHeight="1">
-      <c r="B62" s="155"/>
-      <c r="C62" s="156"/>
-      <c r="D62" s="156"/>
-      <c r="E62" s="156"/>
-      <c r="F62" s="156"/>
-      <c r="G62" s="156"/>
-      <c r="H62" s="156"/>
-      <c r="I62" s="156"/>
-      <c r="J62" s="156"/>
-      <c r="K62" s="156"/>
-      <c r="L62" s="156"/>
-      <c r="M62" s="156"/>
-      <c r="N62" s="156"/>
-      <c r="O62" s="156"/>
-      <c r="P62" s="156"/>
-      <c r="Q62" s="156"/>
-      <c r="R62" s="156"/>
-      <c r="S62" s="156"/>
-      <c r="T62" s="156"/>
-      <c r="U62" s="156"/>
+      <c r="B62" s="132"/>
+      <c r="C62" s="133"/>
+      <c r="D62" s="133"/>
+      <c r="E62" s="133"/>
+      <c r="F62" s="133"/>
+      <c r="G62" s="133"/>
+      <c r="H62" s="133"/>
+      <c r="I62" s="133"/>
+      <c r="J62" s="133"/>
+      <c r="K62" s="133"/>
+      <c r="L62" s="133"/>
+      <c r="M62" s="133"/>
+      <c r="N62" s="133"/>
+      <c r="O62" s="133"/>
+      <c r="P62" s="133"/>
+      <c r="Q62" s="133"/>
+      <c r="R62" s="133"/>
+      <c r="S62" s="133"/>
+      <c r="T62" s="133"/>
+      <c r="U62" s="133"/>
       <c r="V62" s="27"/>
       <c r="W62" s="27"/>
       <c r="X62" s="27"/>
-      <c r="Y62" s="110"/>
-      <c r="Z62" s="110"/>
-      <c r="AA62" s="110"/>
-      <c r="AB62" s="111"/>
-      <c r="AC62" s="110"/>
-      <c r="AD62" s="110"/>
-      <c r="AE62" s="110"/>
-      <c r="AF62" s="110"/>
+      <c r="Y62" s="109"/>
+      <c r="Z62" s="109"/>
+      <c r="AA62" s="109"/>
+      <c r="AB62" s="110"/>
+      <c r="AC62" s="109"/>
+      <c r="AD62" s="109"/>
+      <c r="AE62" s="109"/>
+      <c r="AF62" s="109"/>
       <c r="AG62" s="27"/>
       <c r="AH62" s="27"/>
       <c r="AI62" s="27"/>
@@ -9313,60 +9313,60 @@
       <c r="AN62" s="58"/>
     </row>
     <row r="63" spans="2:40" ht="15" customHeight="1" thickBot="1">
-      <c r="B63" s="113"/>
-      <c r="C63" s="114"/>
-      <c r="D63" s="114"/>
-      <c r="E63" s="114"/>
-      <c r="F63" s="114"/>
-      <c r="G63" s="114"/>
-      <c r="H63" s="114"/>
-      <c r="I63" s="114"/>
-      <c r="J63" s="114"/>
-      <c r="K63" s="114"/>
-      <c r="L63" s="114"/>
-      <c r="M63" s="114"/>
-      <c r="N63" s="114"/>
-      <c r="O63" s="114"/>
-      <c r="P63" s="114"/>
-      <c r="Q63" s="114"/>
-      <c r="R63" s="114"/>
-      <c r="S63" s="114"/>
-      <c r="T63" s="114"/>
-      <c r="U63" s="114"/>
-      <c r="V63" s="115"/>
-      <c r="W63" s="116"/>
-      <c r="X63" s="116"/>
-      <c r="Y63" s="116"/>
-      <c r="Z63" s="116"/>
-      <c r="AA63" s="115"/>
-      <c r="AB63" s="114"/>
-      <c r="AC63" s="114"/>
-      <c r="AD63" s="114"/>
-      <c r="AE63" s="114"/>
-      <c r="AF63" s="114"/>
-      <c r="AG63" s="114"/>
-      <c r="AH63" s="114"/>
-      <c r="AI63" s="114"/>
-      <c r="AJ63" s="114"/>
-      <c r="AK63" s="114"/>
-      <c r="AL63" s="114"/>
-      <c r="AM63" s="114"/>
-      <c r="AN63" s="117"/>
+      <c r="B63" s="112"/>
+      <c r="C63" s="113"/>
+      <c r="D63" s="113"/>
+      <c r="E63" s="113"/>
+      <c r="F63" s="113"/>
+      <c r="G63" s="113"/>
+      <c r="H63" s="113"/>
+      <c r="I63" s="113"/>
+      <c r="J63" s="113"/>
+      <c r="K63" s="113"/>
+      <c r="L63" s="113"/>
+      <c r="M63" s="113"/>
+      <c r="N63" s="113"/>
+      <c r="O63" s="113"/>
+      <c r="P63" s="113"/>
+      <c r="Q63" s="113"/>
+      <c r="R63" s="113"/>
+      <c r="S63" s="113"/>
+      <c r="T63" s="113"/>
+      <c r="U63" s="113"/>
+      <c r="V63" s="114"/>
+      <c r="W63" s="115"/>
+      <c r="X63" s="115"/>
+      <c r="Y63" s="115"/>
+      <c r="Z63" s="115"/>
+      <c r="AA63" s="114"/>
+      <c r="AB63" s="113"/>
+      <c r="AC63" s="113"/>
+      <c r="AD63" s="113"/>
+      <c r="AE63" s="113"/>
+      <c r="AF63" s="113"/>
+      <c r="AG63" s="113"/>
+      <c r="AH63" s="113"/>
+      <c r="AI63" s="113"/>
+      <c r="AJ63" s="113"/>
+      <c r="AK63" s="113"/>
+      <c r="AL63" s="113"/>
+      <c r="AM63" s="113"/>
+      <c r="AN63" s="116"/>
     </row>
     <row r="64" spans="2:40" ht="13.5" customHeight="1">
       <c r="W64" s="1"/>
       <c r="X64" s="1"/>
       <c r="Y64" s="1"/>
-      <c r="Z64" s="118"/>
+      <c r="Z64" s="117"/>
     </row>
     <row r="65" spans="2:40" ht="13.5" customHeight="1">
       <c r="B65" s="2" t="s">
         <v>67</v>
       </c>
       <c r="W65" s="1"/>
-      <c r="X65" s="96"/>
+      <c r="X65" s="95"/>
       <c r="Y65" s="1"/>
-      <c r="Z65" s="119"/>
+      <c r="Z65" s="118"/>
       <c r="AL65" s="5"/>
       <c r="AM65" s="5"/>
       <c r="AN65" s="5"/>
@@ -9375,101 +9375,101 @@
       <c r="B66" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="V66" s="120"/>
+      <c r="V66" s="119"/>
       <c r="W66" s="1"/>
       <c r="X66" s="1"/>
       <c r="Y66" s="1"/>
       <c r="Z66" s="1"/>
-      <c r="AA66" s="120"/>
-      <c r="AB66" s="121"/>
+      <c r="AA66" s="119"/>
+      <c r="AB66" s="120"/>
       <c r="AL66" s="5"/>
       <c r="AM66" s="5"/>
       <c r="AN66" s="5"/>
     </row>
     <row r="67" spans="2:40" ht="13.5" customHeight="1">
-      <c r="C67" s="120"/>
-      <c r="D67" s="120"/>
-      <c r="E67" s="120"/>
-      <c r="F67" s="120"/>
-      <c r="G67" s="120"/>
-      <c r="H67" s="120"/>
-      <c r="I67" s="120"/>
-      <c r="J67" s="120"/>
-      <c r="K67" s="120"/>
-      <c r="L67" s="120"/>
-      <c r="M67" s="120"/>
-      <c r="N67" s="120"/>
-      <c r="O67" s="120"/>
-      <c r="P67" s="120"/>
-      <c r="Q67" s="120"/>
-      <c r="R67" s="120"/>
-      <c r="S67" s="120"/>
-      <c r="U67" s="120"/>
+      <c r="C67" s="119"/>
+      <c r="D67" s="119"/>
+      <c r="E67" s="119"/>
+      <c r="F67" s="119"/>
+      <c r="G67" s="119"/>
+      <c r="H67" s="119"/>
+      <c r="I67" s="119"/>
+      <c r="J67" s="119"/>
+      <c r="K67" s="119"/>
+      <c r="L67" s="119"/>
+      <c r="M67" s="119"/>
+      <c r="N67" s="119"/>
+      <c r="O67" s="119"/>
+      <c r="P67" s="119"/>
+      <c r="Q67" s="119"/>
+      <c r="R67" s="119"/>
+      <c r="S67" s="119"/>
+      <c r="U67" s="119"/>
       <c r="W67" s="1"/>
-      <c r="X67" s="122"/>
-      <c r="Y67" s="122"/>
-      <c r="Z67" s="118"/>
+      <c r="X67" s="121"/>
+      <c r="Y67" s="121"/>
+      <c r="Z67" s="117"/>
       <c r="AL67" s="5"/>
       <c r="AM67" s="5"/>
       <c r="AN67" s="5"/>
     </row>
     <row r="68" spans="2:40" ht="13.5" customHeight="1">
-      <c r="Z68" s="123"/>
+      <c r="Z68" s="122"/>
       <c r="AL68" s="5"/>
       <c r="AM68" s="5"/>
       <c r="AN68" s="5"/>
     </row>
     <row r="69" spans="2:40" ht="13.5" customHeight="1">
-      <c r="Z69" s="123"/>
+      <c r="Z69" s="122"/>
       <c r="AL69" s="5"/>
       <c r="AM69" s="5"/>
       <c r="AN69" s="5"/>
     </row>
     <row r="70" spans="2:40" ht="13.5" customHeight="1">
-      <c r="B70" s="124"/>
-      <c r="C70" s="120"/>
-      <c r="D70" s="120"/>
-      <c r="E70" s="120"/>
-      <c r="F70" s="120"/>
-      <c r="G70" s="120"/>
-      <c r="H70" s="120"/>
-      <c r="I70" s="120"/>
-      <c r="J70" s="120"/>
-      <c r="K70" s="120"/>
-      <c r="L70" s="120"/>
-      <c r="M70" s="120"/>
-      <c r="N70" s="120"/>
-      <c r="O70" s="120"/>
-      <c r="P70" s="120"/>
-      <c r="Q70" s="120"/>
-      <c r="R70" s="120"/>
-      <c r="S70" s="120"/>
-      <c r="U70" s="120"/>
-      <c r="Z70" s="123"/>
+      <c r="B70" s="123"/>
+      <c r="C70" s="119"/>
+      <c r="D70" s="119"/>
+      <c r="E70" s="119"/>
+      <c r="F70" s="119"/>
+      <c r="G70" s="119"/>
+      <c r="H70" s="119"/>
+      <c r="I70" s="119"/>
+      <c r="J70" s="119"/>
+      <c r="K70" s="119"/>
+      <c r="L70" s="119"/>
+      <c r="M70" s="119"/>
+      <c r="N70" s="119"/>
+      <c r="O70" s="119"/>
+      <c r="P70" s="119"/>
+      <c r="Q70" s="119"/>
+      <c r="R70" s="119"/>
+      <c r="S70" s="119"/>
+      <c r="U70" s="119"/>
+      <c r="Z70" s="122"/>
     </row>
     <row r="71" spans="2:40" ht="9.75" customHeight="1">
-      <c r="V71" s="123"/>
-      <c r="W71" s="123"/>
-      <c r="Y71" s="123"/>
-      <c r="Z71" s="123"/>
+      <c r="V71" s="122"/>
+      <c r="W71" s="122"/>
+      <c r="Y71" s="122"/>
+      <c r="Z71" s="122"/>
     </row>
     <row r="72" spans="2:40" ht="13.5" customHeight="1">
-      <c r="V72" s="123"/>
-      <c r="W72" s="123"/>
-      <c r="Y72" s="123"/>
-      <c r="Z72" s="123"/>
+      <c r="V72" s="122"/>
+      <c r="W72" s="122"/>
+      <c r="Y72" s="122"/>
+      <c r="Z72" s="122"/>
     </row>
     <row r="73" spans="2:40" ht="13.5" customHeight="1">
-      <c r="V73" s="123"/>
-      <c r="W73" s="123"/>
-      <c r="Y73" s="123"/>
-      <c r="Z73" s="123"/>
+      <c r="V73" s="122"/>
+      <c r="W73" s="122"/>
+      <c r="Y73" s="122"/>
+      <c r="Z73" s="122"/>
     </row>
     <row r="74" spans="2:40" ht="13.5" customHeight="1">
-      <c r="V74" s="123"/>
-      <c r="W74" s="123"/>
-      <c r="Y74" s="123"/>
-      <c r="Z74" s="123"/>
+      <c r="V74" s="122"/>
+      <c r="W74" s="122"/>
+      <c r="Y74" s="122"/>
+      <c r="Z74" s="122"/>
     </row>
     <row r="75" spans="2:40" ht="13.5" customHeight="1">
       <c r="D75" s="5"/>
@@ -9484,11 +9484,11 @@
       <c r="Q75" s="5"/>
       <c r="R75" s="5"/>
       <c r="S75" s="5"/>
-      <c r="U75" s="123"/>
-      <c r="V75" s="123"/>
-      <c r="W75" s="123"/>
-      <c r="Y75" s="123"/>
-      <c r="Z75" s="123"/>
+      <c r="U75" s="122"/>
+      <c r="V75" s="122"/>
+      <c r="W75" s="122"/>
+      <c r="Y75" s="122"/>
+      <c r="Z75" s="122"/>
     </row>
     <row r="76" spans="2:40" ht="13.5" customHeight="1">
       <c r="D76" s="5"/>
@@ -9503,11 +9503,11 @@
       <c r="Q76" s="5"/>
       <c r="R76" s="5"/>
       <c r="S76" s="5"/>
-      <c r="U76" s="123"/>
-      <c r="V76" s="123"/>
-      <c r="W76" s="123"/>
-      <c r="Y76" s="123"/>
-      <c r="Z76" s="123"/>
+      <c r="U76" s="122"/>
+      <c r="V76" s="122"/>
+      <c r="W76" s="122"/>
+      <c r="Y76" s="122"/>
+      <c r="Z76" s="122"/>
     </row>
     <row r="77" spans="2:40" ht="13.5" customHeight="1">
       <c r="D77" s="5"/>
@@ -9522,11 +9522,11 @@
       <c r="Q77" s="5"/>
       <c r="R77" s="5"/>
       <c r="S77" s="5"/>
-      <c r="U77" s="123"/>
-      <c r="V77" s="123"/>
-      <c r="W77" s="123"/>
-      <c r="Y77" s="123"/>
-      <c r="Z77" s="123"/>
+      <c r="U77" s="122"/>
+      <c r="V77" s="122"/>
+      <c r="W77" s="122"/>
+      <c r="Y77" s="122"/>
+      <c r="Z77" s="122"/>
     </row>
     <row r="78" spans="2:40" ht="13.5" customHeight="1">
       <c r="D78" s="5"/>
@@ -9541,12 +9541,12 @@
       <c r="Q78" s="5"/>
       <c r="R78" s="5"/>
       <c r="S78" s="5"/>
-      <c r="U78" s="123"/>
-      <c r="V78" s="123"/>
-      <c r="W78" s="123"/>
-      <c r="X78" s="123"/>
-      <c r="Y78" s="123"/>
-      <c r="Z78" s="123"/>
+      <c r="U78" s="122"/>
+      <c r="V78" s="122"/>
+      <c r="W78" s="122"/>
+      <c r="X78" s="122"/>
+      <c r="Y78" s="122"/>
+      <c r="Z78" s="122"/>
     </row>
     <row r="79" spans="2:40" ht="13.5" customHeight="1">
       <c r="D79" s="5"/>
@@ -9561,12 +9561,12 @@
       <c r="Q79" s="5"/>
       <c r="R79" s="5"/>
       <c r="S79" s="5"/>
-      <c r="U79" s="123"/>
-      <c r="V79" s="123"/>
-      <c r="W79" s="123"/>
-      <c r="X79" s="123"/>
-      <c r="Y79" s="123"/>
-      <c r="Z79" s="123"/>
+      <c r="U79" s="122"/>
+      <c r="V79" s="122"/>
+      <c r="W79" s="122"/>
+      <c r="X79" s="122"/>
+      <c r="Y79" s="122"/>
+      <c r="Z79" s="122"/>
     </row>
     <row r="80" spans="2:40" ht="13.5" customHeight="1">
       <c r="D80" s="5"/>
@@ -9581,12 +9581,12 @@
       <c r="Q80" s="5"/>
       <c r="R80" s="5"/>
       <c r="S80" s="5"/>
-      <c r="U80" s="123"/>
-      <c r="V80" s="123"/>
-      <c r="W80" s="123"/>
-      <c r="X80" s="123"/>
-      <c r="Y80" s="123"/>
-      <c r="Z80" s="123"/>
+      <c r="U80" s="122"/>
+      <c r="V80" s="122"/>
+      <c r="W80" s="122"/>
+      <c r="X80" s="122"/>
+      <c r="Y80" s="122"/>
+      <c r="Z80" s="122"/>
     </row>
     <row r="81" spans="4:26" ht="13.5" customHeight="1">
       <c r="D81" s="5"/>
@@ -9601,7 +9601,7 @@
       <c r="Q81" s="5"/>
       <c r="R81" s="5"/>
       <c r="S81" s="5"/>
-      <c r="U81" s="123"/>
+      <c r="U81" s="122"/>
     </row>
     <row r="82" spans="4:26" ht="13.5" customHeight="1">
       <c r="D82" s="5"/>
@@ -9616,12 +9616,12 @@
       <c r="Q82" s="5"/>
       <c r="R82" s="5"/>
       <c r="S82" s="5"/>
-      <c r="U82" s="123"/>
-      <c r="V82" s="123"/>
-      <c r="W82" s="123"/>
-      <c r="X82" s="123"/>
-      <c r="Y82" s="123"/>
-      <c r="Z82" s="123"/>
+      <c r="U82" s="122"/>
+      <c r="V82" s="122"/>
+      <c r="W82" s="122"/>
+      <c r="X82" s="122"/>
+      <c r="Y82" s="122"/>
+      <c r="Z82" s="122"/>
     </row>
     <row r="83" spans="4:26" ht="13.5" customHeight="1">
       <c r="D83" s="5"/>
@@ -9636,12 +9636,12 @@
       <c r="Q83" s="5"/>
       <c r="R83" s="5"/>
       <c r="S83" s="5"/>
-      <c r="U83" s="123"/>
-      <c r="V83" s="123"/>
-      <c r="W83" s="123"/>
-      <c r="X83" s="123"/>
-      <c r="Y83" s="123"/>
-      <c r="Z83" s="123"/>
+      <c r="U83" s="122"/>
+      <c r="V83" s="122"/>
+      <c r="W83" s="122"/>
+      <c r="X83" s="122"/>
+      <c r="Y83" s="122"/>
+      <c r="Z83" s="122"/>
     </row>
     <row r="84" spans="4:26" ht="13.5" customHeight="1">
       <c r="D84" s="5"/>
@@ -9656,22 +9656,22 @@
       <c r="Q84" s="5"/>
       <c r="R84" s="5"/>
       <c r="S84" s="5"/>
-      <c r="U84" s="123"/>
-      <c r="V84" s="123"/>
-      <c r="W84" s="123"/>
-      <c r="X84" s="123"/>
-      <c r="Y84" s="123"/>
-      <c r="Z84" s="123"/>
+      <c r="U84" s="122"/>
+      <c r="V84" s="122"/>
+      <c r="W84" s="122"/>
+      <c r="X84" s="122"/>
+      <c r="Y84" s="122"/>
+      <c r="Z84" s="122"/>
     </row>
     <row r="85" spans="4:26" ht="13.5" customHeight="1">
       <c r="D85" s="5"/>
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
-      <c r="V85" s="123"/>
-      <c r="W85" s="123"/>
-      <c r="X85" s="123"/>
-      <c r="Y85" s="123"/>
-      <c r="Z85" s="123"/>
+      <c r="V85" s="122"/>
+      <c r="W85" s="122"/>
+      <c r="X85" s="122"/>
+      <c r="Y85" s="122"/>
+      <c r="Z85" s="122"/>
     </row>
     <row r="86" spans="4:26" ht="13.5" customHeight="1">
       <c r="D86" s="5"/>
@@ -9686,12 +9686,12 @@
       <c r="Q86" s="5"/>
       <c r="R86" s="5"/>
       <c r="S86" s="5"/>
-      <c r="U86" s="123"/>
-      <c r="V86" s="123"/>
-      <c r="W86" s="123"/>
-      <c r="X86" s="123"/>
-      <c r="Y86" s="123"/>
-      <c r="Z86" s="123"/>
+      <c r="U86" s="122"/>
+      <c r="V86" s="122"/>
+      <c r="W86" s="122"/>
+      <c r="X86" s="122"/>
+      <c r="Y86" s="122"/>
+      <c r="Z86" s="122"/>
     </row>
     <row r="87" spans="4:26" ht="14.15" customHeight="1">
       <c r="D87" s="5"/>
@@ -9706,7 +9706,7 @@
       <c r="Q87" s="5"/>
       <c r="R87" s="5"/>
       <c r="S87" s="5"/>
-      <c r="U87" s="123"/>
+      <c r="U87" s="122"/>
     </row>
     <row r="88" spans="4:26" ht="14.15" customHeight="1">
       <c r="D88" s="5"/>
@@ -9721,10 +9721,10 @@
       <c r="Q88" s="5"/>
       <c r="R88" s="5"/>
       <c r="S88" s="5"/>
-      <c r="U88" s="123"/>
-      <c r="V88" s="123"/>
-      <c r="W88" s="123"/>
-      <c r="X88" s="123"/>
+      <c r="U88" s="122"/>
+      <c r="V88" s="122"/>
+      <c r="W88" s="122"/>
+      <c r="X88" s="122"/>
     </row>
     <row r="89" spans="4:26" ht="14.15" customHeight="1">
       <c r="D89" s="5"/>
@@ -9739,10 +9739,10 @@
       <c r="Q89" s="5"/>
       <c r="R89" s="5"/>
       <c r="S89" s="5"/>
-      <c r="U89" s="123"/>
-      <c r="V89" s="123"/>
-      <c r="W89" s="123"/>
-      <c r="X89" s="123"/>
+      <c r="U89" s="122"/>
+      <c r="V89" s="122"/>
+      <c r="W89" s="122"/>
+      <c r="X89" s="122"/>
     </row>
     <row r="90" spans="4:26" ht="14.15" customHeight="1">
       <c r="D90" s="5"/>
@@ -9757,19 +9757,19 @@
       <c r="Q90" s="5"/>
       <c r="R90" s="5"/>
       <c r="S90" s="5"/>
-      <c r="U90" s="123"/>
-      <c r="V90" s="123"/>
-      <c r="W90" s="123"/>
-      <c r="X90" s="123"/>
-      <c r="Y90" s="123"/>
-      <c r="Z90" s="123"/>
+      <c r="U90" s="122"/>
+      <c r="V90" s="122"/>
+      <c r="W90" s="122"/>
+      <c r="X90" s="122"/>
+      <c r="Y90" s="122"/>
+      <c r="Z90" s="122"/>
     </row>
     <row r="91" spans="4:26" ht="14.15" customHeight="1">
-      <c r="V91" s="123"/>
-      <c r="W91" s="123"/>
-      <c r="X91" s="123"/>
-      <c r="Y91" s="123"/>
-      <c r="Z91" s="123"/>
+      <c r="V91" s="122"/>
+      <c r="W91" s="122"/>
+      <c r="X91" s="122"/>
+      <c r="Y91" s="122"/>
+      <c r="Z91" s="122"/>
     </row>
     <row r="92" spans="4:26" ht="14.15" customHeight="1">
       <c r="D92" s="5"/>
@@ -9784,12 +9784,12 @@
       <c r="Q92" s="5"/>
       <c r="R92" s="5"/>
       <c r="S92" s="5"/>
-      <c r="U92" s="123"/>
-      <c r="V92" s="123"/>
-      <c r="W92" s="123"/>
-      <c r="X92" s="123"/>
-      <c r="Y92" s="123"/>
-      <c r="Z92" s="123"/>
+      <c r="U92" s="122"/>
+      <c r="V92" s="122"/>
+      <c r="W92" s="122"/>
+      <c r="X92" s="122"/>
+      <c r="Y92" s="122"/>
+      <c r="Z92" s="122"/>
     </row>
     <row r="93" spans="4:26" ht="14.15" customHeight="1">
       <c r="D93" s="5"/>
@@ -9804,12 +9804,12 @@
       <c r="Q93" s="5"/>
       <c r="R93" s="5"/>
       <c r="S93" s="5"/>
-      <c r="U93" s="123"/>
-      <c r="V93" s="123"/>
-      <c r="W93" s="123"/>
-      <c r="X93" s="123"/>
-      <c r="Y93" s="123"/>
-      <c r="Z93" s="123"/>
+      <c r="U93" s="122"/>
+      <c r="V93" s="122"/>
+      <c r="W93" s="122"/>
+      <c r="X93" s="122"/>
+      <c r="Y93" s="122"/>
+      <c r="Z93" s="122"/>
     </row>
     <row r="94" spans="4:26" ht="14.15" customHeight="1">
       <c r="D94" s="5"/>
@@ -9824,12 +9824,12 @@
       <c r="Q94" s="5"/>
       <c r="R94" s="5"/>
       <c r="S94" s="5"/>
-      <c r="U94" s="123"/>
-      <c r="V94" s="123"/>
-      <c r="W94" s="123"/>
-      <c r="X94" s="123"/>
-      <c r="Y94" s="123"/>
-      <c r="Z94" s="123"/>
+      <c r="U94" s="122"/>
+      <c r="V94" s="122"/>
+      <c r="W94" s="122"/>
+      <c r="X94" s="122"/>
+      <c r="Y94" s="122"/>
+      <c r="Z94" s="122"/>
     </row>
     <row r="95" spans="4:26" ht="14.15" customHeight="1">
       <c r="D95" s="5"/>
@@ -9844,12 +9844,12 @@
       <c r="Q95" s="5"/>
       <c r="R95" s="5"/>
       <c r="S95" s="5"/>
-      <c r="U95" s="123"/>
-      <c r="V95" s="123"/>
-      <c r="W95" s="123"/>
-      <c r="X95" s="123"/>
-      <c r="Y95" s="123"/>
-      <c r="Z95" s="123"/>
+      <c r="U95" s="122"/>
+      <c r="V95" s="122"/>
+      <c r="W95" s="122"/>
+      <c r="X95" s="122"/>
+      <c r="Y95" s="122"/>
+      <c r="Z95" s="122"/>
     </row>
     <row r="96" spans="4:26" ht="14.15" customHeight="1">
       <c r="D96" s="5"/>
@@ -9864,12 +9864,12 @@
       <c r="Q96" s="5"/>
       <c r="R96" s="5"/>
       <c r="S96" s="5"/>
-      <c r="U96" s="123"/>
-      <c r="V96" s="123"/>
-      <c r="W96" s="123"/>
-      <c r="X96" s="123"/>
-      <c r="Y96" s="123"/>
-      <c r="Z96" s="123"/>
+      <c r="U96" s="122"/>
+      <c r="V96" s="122"/>
+      <c r="W96" s="122"/>
+      <c r="X96" s="122"/>
+      <c r="Y96" s="122"/>
+      <c r="Z96" s="122"/>
     </row>
     <row r="97" spans="4:29" ht="14.15" customHeight="1">
       <c r="D97" s="5"/>
@@ -9884,12 +9884,12 @@
       <c r="Q97" s="5"/>
       <c r="R97" s="5"/>
       <c r="S97" s="5"/>
-      <c r="U97" s="123"/>
-      <c r="V97" s="123"/>
-      <c r="W97" s="123"/>
-      <c r="X97" s="123"/>
-      <c r="Y97" s="123"/>
-      <c r="Z97" s="123"/>
+      <c r="U97" s="122"/>
+      <c r="V97" s="122"/>
+      <c r="W97" s="122"/>
+      <c r="X97" s="122"/>
+      <c r="Y97" s="122"/>
+      <c r="Z97" s="122"/>
     </row>
     <row r="98" spans="4:29" ht="14.15" customHeight="1">
       <c r="D98" s="5"/>
@@ -9904,12 +9904,12 @@
       <c r="Q98" s="5"/>
       <c r="R98" s="5"/>
       <c r="S98" s="5"/>
-      <c r="U98" s="123"/>
-      <c r="V98" s="123"/>
-      <c r="W98" s="123"/>
-      <c r="X98" s="123"/>
-      <c r="Y98" s="123"/>
-      <c r="Z98" s="123"/>
+      <c r="U98" s="122"/>
+      <c r="V98" s="122"/>
+      <c r="W98" s="122"/>
+      <c r="X98" s="122"/>
+      <c r="Y98" s="122"/>
+      <c r="Z98" s="122"/>
     </row>
     <row r="99" spans="4:29" ht="14.15" customHeight="1">
       <c r="D99" s="5"/>
@@ -9924,12 +9924,12 @@
       <c r="Q99" s="5"/>
       <c r="R99" s="5"/>
       <c r="S99" s="5"/>
-      <c r="U99" s="123"/>
-      <c r="V99" s="123"/>
-      <c r="W99" s="123"/>
-      <c r="X99" s="123"/>
-      <c r="Y99" s="123"/>
-      <c r="Z99" s="123"/>
+      <c r="U99" s="122"/>
+      <c r="V99" s="122"/>
+      <c r="W99" s="122"/>
+      <c r="X99" s="122"/>
+      <c r="Y99" s="122"/>
+      <c r="Z99" s="122"/>
     </row>
     <row r="100" spans="4:29" ht="14.15" customHeight="1">
       <c r="D100" s="5"/>
@@ -9944,9 +9944,9 @@
       <c r="Q100" s="5"/>
       <c r="R100" s="5"/>
       <c r="S100" s="5"/>
-      <c r="U100" s="123"/>
-      <c r="AB100" s="121"/>
-      <c r="AC100" s="120"/>
+      <c r="U100" s="122"/>
+      <c r="AB100" s="120"/>
+      <c r="AC100" s="119"/>
     </row>
     <row r="101" spans="4:29" ht="14.15" customHeight="1">
       <c r="D101" s="5"/>
@@ -9961,12 +9961,12 @@
       <c r="Q101" s="5"/>
       <c r="R101" s="5"/>
       <c r="S101" s="5"/>
-      <c r="U101" s="123"/>
-      <c r="V101" s="123"/>
-      <c r="W101" s="123"/>
-      <c r="X101" s="123"/>
-      <c r="Y101" s="123"/>
-      <c r="Z101" s="123"/>
+      <c r="U101" s="122"/>
+      <c r="V101" s="122"/>
+      <c r="W101" s="122"/>
+      <c r="X101" s="122"/>
+      <c r="Y101" s="122"/>
+      <c r="Z101" s="122"/>
     </row>
     <row r="102" spans="4:29" ht="14.15" customHeight="1">
       <c r="D102" s="5"/>
@@ -9981,12 +9981,12 @@
       <c r="Q102" s="5"/>
       <c r="R102" s="5"/>
       <c r="S102" s="5"/>
-      <c r="U102" s="123"/>
-      <c r="V102" s="123"/>
-      <c r="W102" s="123"/>
-      <c r="X102" s="123"/>
-      <c r="Y102" s="123"/>
-      <c r="Z102" s="123"/>
+      <c r="U102" s="122"/>
+      <c r="V102" s="122"/>
+      <c r="W102" s="122"/>
+      <c r="X102" s="122"/>
+      <c r="Y102" s="122"/>
+      <c r="Z102" s="122"/>
     </row>
     <row r="103" spans="4:29" ht="14.15" customHeight="1">
       <c r="D103" s="5"/>
@@ -10001,19 +10001,19 @@
       <c r="Q103" s="5"/>
       <c r="R103" s="5"/>
       <c r="S103" s="5"/>
-      <c r="U103" s="123"/>
-      <c r="V103" s="123"/>
-      <c r="W103" s="123"/>
-      <c r="X103" s="123"/>
-      <c r="Y103" s="123"/>
-      <c r="Z103" s="123"/>
+      <c r="U103" s="122"/>
+      <c r="V103" s="122"/>
+      <c r="W103" s="122"/>
+      <c r="X103" s="122"/>
+      <c r="Y103" s="122"/>
+      <c r="Z103" s="122"/>
     </row>
     <row r="104" spans="4:29" ht="14.15" customHeight="1">
-      <c r="V104" s="123"/>
-      <c r="W104" s="123"/>
-      <c r="X104" s="123"/>
-      <c r="Y104" s="123"/>
-      <c r="Z104" s="123"/>
+      <c r="V104" s="122"/>
+      <c r="W104" s="122"/>
+      <c r="X104" s="122"/>
+      <c r="Y104" s="122"/>
+      <c r="Z104" s="122"/>
     </row>
     <row r="105" spans="4:29" ht="19.5" customHeight="1">
       <c r="D105" s="5"/>
@@ -10028,12 +10028,12 @@
       <c r="Q105" s="5"/>
       <c r="R105" s="5"/>
       <c r="S105" s="5"/>
-      <c r="U105" s="123"/>
-      <c r="V105" s="123"/>
-      <c r="W105" s="123"/>
-      <c r="X105" s="123"/>
-      <c r="Y105" s="123"/>
-      <c r="Z105" s="123"/>
+      <c r="U105" s="122"/>
+      <c r="V105" s="122"/>
+      <c r="W105" s="122"/>
+      <c r="X105" s="122"/>
+      <c r="Y105" s="122"/>
+      <c r="Z105" s="122"/>
     </row>
     <row r="106" spans="4:29" ht="14.15" customHeight="1">
       <c r="D106" s="5"/>
@@ -10048,12 +10048,12 @@
       <c r="Q106" s="5"/>
       <c r="R106" s="5"/>
       <c r="S106" s="5"/>
-      <c r="U106" s="123"/>
-      <c r="V106" s="123"/>
-      <c r="W106" s="123"/>
-      <c r="X106" s="123"/>
-      <c r="Y106" s="123"/>
-      <c r="Z106" s="123"/>
+      <c r="U106" s="122"/>
+      <c r="V106" s="122"/>
+      <c r="W106" s="122"/>
+      <c r="X106" s="122"/>
+      <c r="Y106" s="122"/>
+      <c r="Z106" s="122"/>
     </row>
     <row r="107" spans="4:29" ht="14.15" customHeight="1">
       <c r="D107" s="5"/>
@@ -10068,12 +10068,12 @@
       <c r="Q107" s="5"/>
       <c r="R107" s="5"/>
       <c r="S107" s="5"/>
-      <c r="U107" s="123"/>
-      <c r="V107" s="123"/>
-      <c r="W107" s="123"/>
-      <c r="X107" s="123"/>
-      <c r="Y107" s="123"/>
-      <c r="Z107" s="123"/>
+      <c r="U107" s="122"/>
+      <c r="V107" s="122"/>
+      <c r="W107" s="122"/>
+      <c r="X107" s="122"/>
+      <c r="Y107" s="122"/>
+      <c r="Z107" s="122"/>
     </row>
     <row r="108" spans="4:29" ht="14.15" customHeight="1">
       <c r="D108" s="5"/>
@@ -10088,12 +10088,12 @@
       <c r="Q108" s="5"/>
       <c r="R108" s="5"/>
       <c r="S108" s="5"/>
-      <c r="U108" s="123"/>
-      <c r="V108" s="123"/>
-      <c r="W108" s="123"/>
-      <c r="X108" s="123"/>
-      <c r="Y108" s="123"/>
-      <c r="Z108" s="123"/>
+      <c r="U108" s="122"/>
+      <c r="V108" s="122"/>
+      <c r="W108" s="122"/>
+      <c r="X108" s="122"/>
+      <c r="Y108" s="122"/>
+      <c r="Z108" s="122"/>
     </row>
     <row r="109" spans="4:29" ht="14.15" customHeight="1">
       <c r="D109" s="5"/>
@@ -10108,12 +10108,12 @@
       <c r="Q109" s="5"/>
       <c r="R109" s="5"/>
       <c r="S109" s="5"/>
-      <c r="U109" s="123"/>
-      <c r="V109" s="123"/>
-      <c r="W109" s="123"/>
-      <c r="X109" s="123"/>
-      <c r="Y109" s="123"/>
-      <c r="Z109" s="123"/>
+      <c r="U109" s="122"/>
+      <c r="V109" s="122"/>
+      <c r="W109" s="122"/>
+      <c r="X109" s="122"/>
+      <c r="Y109" s="122"/>
+      <c r="Z109" s="122"/>
     </row>
     <row r="110" spans="4:29" ht="14.15" customHeight="1">
       <c r="D110" s="5"/>
@@ -10128,12 +10128,12 @@
       <c r="Q110" s="5"/>
       <c r="R110" s="5"/>
       <c r="S110" s="5"/>
-      <c r="U110" s="123"/>
-      <c r="V110" s="123"/>
-      <c r="W110" s="123"/>
-      <c r="X110" s="123"/>
-      <c r="Y110" s="123"/>
-      <c r="Z110" s="123"/>
+      <c r="U110" s="122"/>
+      <c r="V110" s="122"/>
+      <c r="W110" s="122"/>
+      <c r="X110" s="122"/>
+      <c r="Y110" s="122"/>
+      <c r="Z110" s="122"/>
     </row>
     <row r="111" spans="4:29" ht="14.15" customHeight="1"/>
     <row r="112" spans="4:29" ht="14.15" customHeight="1"/>
@@ -10145,51 +10145,51 @@
     <row r="118" spans="35:37" ht="14.15" customHeight="1"/>
     <row r="119" spans="35:37" ht="14.15" customHeight="1"/>
     <row r="120" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI120" s="125"/>
-      <c r="AJ120" s="125"/>
-      <c r="AK120" s="125"/>
+      <c r="AI120" s="124"/>
+      <c r="AJ120" s="124"/>
+      <c r="AK120" s="124"/>
     </row>
     <row r="121" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI121" s="125"/>
-      <c r="AJ121" s="125"/>
-      <c r="AK121" s="125"/>
+      <c r="AI121" s="124"/>
+      <c r="AJ121" s="124"/>
+      <c r="AK121" s="124"/>
     </row>
     <row r="122" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI122" s="125"/>
-      <c r="AJ122" s="125"/>
-      <c r="AK122" s="125"/>
+      <c r="AI122" s="124"/>
+      <c r="AJ122" s="124"/>
+      <c r="AK122" s="124"/>
     </row>
     <row r="123" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI123" s="125"/>
-      <c r="AJ123" s="125"/>
-      <c r="AK123" s="125"/>
+      <c r="AI123" s="124"/>
+      <c r="AJ123" s="124"/>
+      <c r="AK123" s="124"/>
     </row>
     <row r="124" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI124" s="125"/>
-      <c r="AJ124" s="125"/>
-      <c r="AK124" s="125"/>
+      <c r="AI124" s="124"/>
+      <c r="AJ124" s="124"/>
+      <c r="AK124" s="124"/>
     </row>
     <row r="125" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI125" s="125"/>
-      <c r="AJ125" s="125"/>
-      <c r="AK125" s="125"/>
+      <c r="AI125" s="124"/>
+      <c r="AJ125" s="124"/>
+      <c r="AK125" s="124"/>
     </row>
     <row r="126" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI126" s="125"/>
-      <c r="AJ126" s="125"/>
-      <c r="AK126" s="125"/>
+      <c r="AI126" s="124"/>
+      <c r="AJ126" s="124"/>
+      <c r="AK126" s="124"/>
     </row>
     <row r="127" spans="35:37" ht="14.15" customHeight="1">
-      <c r="AI127" s="125"/>
-      <c r="AJ127" s="125"/>
-      <c r="AK127" s="125"/>
+      <c r="AI127" s="124"/>
+      <c r="AJ127" s="124"/>
+      <c r="AK127" s="124"/>
     </row>
     <row r="128" spans="35:37">
-      <c r="AI128" s="125"/>
-      <c r="AJ128" s="125"/>
-      <c r="AK128" s="125"/>
-    </row>
-    <row r="129" spans="2:34" s="125" customFormat="1" ht="12.75" customHeight="1">
+      <c r="AI128" s="124"/>
+      <c r="AJ128" s="124"/>
+      <c r="AK128" s="124"/>
+    </row>
+    <row r="129" spans="2:34" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="C129" s="2"/>
       <c r="D129" s="2"/>
       <c r="E129" s="2"/>
@@ -10223,7 +10223,7 @@
       <c r="AG129" s="2"/>
       <c r="AH129" s="2"/>
     </row>
-    <row r="130" spans="2:34" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="130" spans="2:34" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="C130" s="2"/>
       <c r="D130" s="2"/>
       <c r="E130" s="2"/>
@@ -10257,7 +10257,7 @@
       <c r="AG130" s="2"/>
       <c r="AH130" s="2"/>
     </row>
-    <row r="131" spans="2:34" s="125" customFormat="1">
+    <row r="131" spans="2:34" s="124" customFormat="1">
       <c r="C131" s="2"/>
       <c r="D131" s="2"/>
       <c r="E131" s="2"/>
@@ -10291,7 +10291,7 @@
       <c r="AG131" s="2"/>
       <c r="AH131" s="2"/>
     </row>
-    <row r="132" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="132" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
       <c r="D132" s="2"/>
@@ -10326,7 +10326,7 @@
       <c r="AG132" s="2"/>
       <c r="AH132" s="2"/>
     </row>
-    <row r="133" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="133" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
       <c r="D133" s="2"/>
@@ -10361,7 +10361,7 @@
       <c r="AG133" s="2"/>
       <c r="AH133" s="2"/>
     </row>
-    <row r="134" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="134" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
       <c r="D134" s="2"/>
@@ -10396,7 +10396,7 @@
       <c r="AG134" s="2"/>
       <c r="AH134" s="2"/>
     </row>
-    <row r="135" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="135" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
       <c r="D135" s="2"/>
@@ -10431,7 +10431,7 @@
       <c r="AG135" s="2"/>
       <c r="AH135" s="2"/>
     </row>
-    <row r="136" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="136" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
       <c r="D136" s="2"/>
@@ -10466,7 +10466,7 @@
       <c r="AG136" s="2"/>
       <c r="AH136" s="2"/>
     </row>
-    <row r="137" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="137" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
       <c r="D137" s="2"/>
@@ -10501,7 +10501,7 @@
       <c r="AG137" s="2"/>
       <c r="AH137" s="2"/>
     </row>
-    <row r="138" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="138" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
       <c r="D138" s="2"/>
@@ -10536,7 +10536,7 @@
       <c r="AG138" s="2"/>
       <c r="AH138" s="2"/>
     </row>
-    <row r="139" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="139" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
       <c r="D139" s="2"/>
@@ -10571,7 +10571,7 @@
       <c r="AG139" s="2"/>
       <c r="AH139" s="2"/>
     </row>
-    <row r="140" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="140" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
       <c r="D140" s="2"/>
@@ -10606,7 +10606,7 @@
       <c r="AG140" s="2"/>
       <c r="AH140" s="2"/>
     </row>
-    <row r="141" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="141" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
       <c r="D141" s="2"/>
@@ -10641,7 +10641,7 @@
       <c r="AG141" s="2"/>
       <c r="AH141" s="2"/>
     </row>
-    <row r="142" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="142" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
       <c r="D142" s="2"/>
@@ -10676,7 +10676,7 @@
       <c r="AG142" s="2"/>
       <c r="AH142" s="2"/>
     </row>
-    <row r="143" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="143" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
       <c r="D143" s="2"/>
@@ -10711,7 +10711,7 @@
       <c r="AG143" s="2"/>
       <c r="AH143" s="2"/>
     </row>
-    <row r="144" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="144" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
       <c r="D144" s="2"/>
@@ -10746,7 +10746,7 @@
       <c r="AG144" s="2"/>
       <c r="AH144" s="2"/>
     </row>
-    <row r="145" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="145" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
       <c r="D145" s="2"/>
@@ -10781,7 +10781,7 @@
       <c r="AG145" s="2"/>
       <c r="AH145" s="2"/>
     </row>
-    <row r="146" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="146" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
       <c r="D146" s="2"/>
@@ -10816,7 +10816,7 @@
       <c r="AG146" s="2"/>
       <c r="AH146" s="2"/>
     </row>
-    <row r="147" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="147" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
       <c r="D147" s="2"/>
@@ -10851,7 +10851,7 @@
       <c r="AG147" s="2"/>
       <c r="AH147" s="2"/>
     </row>
-    <row r="148" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="148" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
       <c r="D148" s="2"/>
@@ -10886,7 +10886,7 @@
       <c r="AG148" s="2"/>
       <c r="AH148" s="2"/>
     </row>
-    <row r="149" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="149" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
       <c r="D149" s="2"/>
@@ -10921,7 +10921,7 @@
       <c r="AG149" s="2"/>
       <c r="AH149" s="2"/>
     </row>
-    <row r="150" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="150" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
       <c r="D150" s="2"/>
@@ -10956,7 +10956,7 @@
       <c r="AG150" s="2"/>
       <c r="AH150" s="2"/>
     </row>
-    <row r="151" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="151" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
       <c r="D151" s="2"/>
@@ -10991,7 +10991,7 @@
       <c r="AG151" s="2"/>
       <c r="AH151" s="2"/>
     </row>
-    <row r="152" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="152" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
       <c r="D152" s="2"/>
@@ -11026,7 +11026,7 @@
       <c r="AG152" s="2"/>
       <c r="AH152" s="2"/>
     </row>
-    <row r="153" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="153" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
       <c r="D153" s="2"/>
@@ -11061,7 +11061,7 @@
       <c r="AG153" s="2"/>
       <c r="AH153" s="2"/>
     </row>
-    <row r="154" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="154" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
       <c r="D154" s="2"/>
@@ -11096,7 +11096,7 @@
       <c r="AG154" s="2"/>
       <c r="AH154" s="2"/>
     </row>
-    <row r="155" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="155" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
       <c r="D155" s="2"/>
@@ -11131,7 +11131,7 @@
       <c r="AG155" s="2"/>
       <c r="AH155" s="2"/>
     </row>
-    <row r="156" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="156" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
       <c r="D156" s="2"/>
@@ -11166,7 +11166,7 @@
       <c r="AG156" s="2"/>
       <c r="AH156" s="2"/>
     </row>
-    <row r="157" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="157" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
       <c r="D157" s="2"/>
@@ -11201,7 +11201,7 @@
       <c r="AG157" s="2"/>
       <c r="AH157" s="2"/>
     </row>
-    <row r="158" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="158" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
       <c r="D158" s="2"/>
@@ -11236,7 +11236,7 @@
       <c r="AG158" s="2"/>
       <c r="AH158" s="2"/>
     </row>
-    <row r="159" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="159" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
       <c r="D159" s="2"/>
@@ -11271,7 +11271,7 @@
       <c r="AG159" s="2"/>
       <c r="AH159" s="2"/>
     </row>
-    <row r="160" spans="2:34" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="160" spans="2:34" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
       <c r="D160" s="2"/>
@@ -11306,7 +11306,7 @@
       <c r="AG160" s="2"/>
       <c r="AH160" s="2"/>
     </row>
-    <row r="161" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="161" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
       <c r="D161" s="2"/>
@@ -11341,7 +11341,7 @@
       <c r="AG161" s="2"/>
       <c r="AH161" s="2"/>
     </row>
-    <row r="162" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="162" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
       <c r="D162" s="2"/>
@@ -11376,7 +11376,7 @@
       <c r="AG162" s="2"/>
       <c r="AH162" s="2"/>
     </row>
-    <row r="163" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="163" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
       <c r="D163" s="2"/>
@@ -11411,7 +11411,7 @@
       <c r="AG163" s="2"/>
       <c r="AH163" s="2"/>
     </row>
-    <row r="164" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="164" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
       <c r="D164" s="2"/>
@@ -11446,7 +11446,7 @@
       <c r="AG164" s="2"/>
       <c r="AH164" s="2"/>
     </row>
-    <row r="165" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="165" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
       <c r="D165" s="2"/>
@@ -11481,7 +11481,7 @@
       <c r="AG165" s="2"/>
       <c r="AH165" s="2"/>
     </row>
-    <row r="166" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="166" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
       <c r="D166" s="2"/>
@@ -11516,7 +11516,7 @@
       <c r="AG166" s="2"/>
       <c r="AH166" s="2"/>
     </row>
-    <row r="167" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="167" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
       <c r="D167" s="2"/>
@@ -11551,7 +11551,7 @@
       <c r="AG167" s="2"/>
       <c r="AH167" s="2"/>
     </row>
-    <row r="168" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="168" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
       <c r="D168" s="2"/>
@@ -11586,7 +11586,7 @@
       <c r="AG168" s="2"/>
       <c r="AH168" s="2"/>
     </row>
-    <row r="169" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="169" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
       <c r="D169" s="2"/>
@@ -11621,7 +11621,7 @@
       <c r="AG169" s="2"/>
       <c r="AH169" s="2"/>
     </row>
-    <row r="170" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="170" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
       <c r="D170" s="2"/>
@@ -11656,7 +11656,7 @@
       <c r="AG170" s="2"/>
       <c r="AH170" s="2"/>
     </row>
-    <row r="171" spans="2:37" s="125" customFormat="1" ht="24">
+    <row r="171" spans="2:37" s="124" customFormat="1" ht="24">
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
       <c r="D171" s="2"/>
@@ -11690,11 +11690,11 @@
       <c r="AF171" s="2"/>
       <c r="AG171" s="2"/>
       <c r="AH171" s="2"/>
-      <c r="AI171" s="126"/>
-      <c r="AJ171" s="126"/>
-      <c r="AK171" s="126"/>
-    </row>
-    <row r="172" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+      <c r="AI171" s="125"/>
+      <c r="AJ171" s="125"/>
+      <c r="AK171" s="125"/>
+    </row>
+    <row r="172" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
       <c r="D172" s="2"/>
@@ -11729,7 +11729,7 @@
       <c r="AG172" s="2"/>
       <c r="AH172" s="2"/>
     </row>
-    <row r="173" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="173" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B173" s="2"/>
       <c r="C173" s="2"/>
       <c r="D173" s="2"/>
@@ -11764,7 +11764,7 @@
       <c r="AG173" s="2"/>
       <c r="AH173" s="2"/>
     </row>
-    <row r="174" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="174" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B174" s="2"/>
       <c r="C174" s="2"/>
       <c r="D174" s="2"/>
@@ -11799,7 +11799,7 @@
       <c r="AG174" s="2"/>
       <c r="AH174" s="2"/>
     </row>
-    <row r="175" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="175" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B175" s="2"/>
       <c r="C175" s="2"/>
       <c r="D175" s="2"/>
@@ -11834,7 +11834,7 @@
       <c r="AG175" s="2"/>
       <c r="AH175" s="2"/>
     </row>
-    <row r="176" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="176" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B176" s="2"/>
       <c r="C176" s="2"/>
       <c r="D176" s="2"/>
@@ -11869,7 +11869,7 @@
       <c r="AG176" s="2"/>
       <c r="AH176" s="2"/>
     </row>
-    <row r="177" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="177" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
       <c r="D177" s="2"/>
@@ -11904,7 +11904,7 @@
       <c r="AG177" s="2"/>
       <c r="AH177" s="2"/>
     </row>
-    <row r="178" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="178" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
       <c r="D178" s="2"/>
@@ -11939,7 +11939,7 @@
       <c r="AG178" s="2"/>
       <c r="AH178" s="2"/>
     </row>
-    <row r="179" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="179" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
       <c r="D179" s="2"/>
@@ -11974,7 +11974,7 @@
       <c r="AG179" s="2"/>
       <c r="AH179" s="2"/>
     </row>
-    <row r="180" spans="2:37" s="126" customFormat="1" ht="20.25" customHeight="1">
+    <row r="180" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
       <c r="D180" s="2"/>
@@ -12008,11 +12008,11 @@
       <c r="AF180" s="2"/>
       <c r="AG180" s="2"/>
       <c r="AH180" s="2"/>
-      <c r="AI180" s="125"/>
-      <c r="AJ180" s="125"/>
-      <c r="AK180" s="125"/>
-    </row>
-    <row r="181" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+      <c r="AI180" s="124"/>
+      <c r="AJ180" s="124"/>
+      <c r="AK180" s="124"/>
+    </row>
+    <row r="181" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
       <c r="D181" s="2"/>
@@ -12047,7 +12047,7 @@
       <c r="AG181" s="2"/>
       <c r="AH181" s="2"/>
     </row>
-    <row r="182" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="182" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
       <c r="D182" s="2"/>
@@ -12082,7 +12082,7 @@
       <c r="AG182" s="2"/>
       <c r="AH182" s="2"/>
     </row>
-    <row r="183" spans="2:37" s="125" customFormat="1">
+    <row r="183" spans="2:37" s="124" customFormat="1">
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
       <c r="D183" s="2"/>
@@ -12117,7 +12117,7 @@
       <c r="AG183" s="2"/>
       <c r="AH183" s="2"/>
     </row>
-    <row r="184" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="184" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
       <c r="D184" s="2"/>
@@ -12152,7 +12152,7 @@
       <c r="AG184" s="2"/>
       <c r="AH184" s="2"/>
     </row>
-    <row r="185" spans="2:37" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="185" spans="2:37" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
       <c r="D185" s="2"/>
@@ -12187,7 +12187,7 @@
       <c r="AG185" s="2"/>
       <c r="AH185" s="2"/>
     </row>
-    <row r="186" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="186" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B186" s="2"/>
       <c r="C186" s="2"/>
       <c r="D186" s="2"/>
@@ -12222,7 +12222,7 @@
       <c r="AG186" s="2"/>
       <c r="AH186" s="2"/>
     </row>
-    <row r="187" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="187" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
       <c r="D187" s="2"/>
@@ -12257,7 +12257,7 @@
       <c r="AG187" s="2"/>
       <c r="AH187" s="2"/>
     </row>
-    <row r="188" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="188" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B188" s="2"/>
       <c r="C188" s="2"/>
       <c r="D188" s="2"/>
@@ -12292,7 +12292,7 @@
       <c r="AG188" s="2"/>
       <c r="AH188" s="2"/>
     </row>
-    <row r="189" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="189" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
       <c r="D189" s="2"/>
@@ -12327,7 +12327,7 @@
       <c r="AG189" s="2"/>
       <c r="AH189" s="2"/>
     </row>
-    <row r="190" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="190" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B190" s="2"/>
       <c r="C190" s="2"/>
       <c r="D190" s="2"/>
@@ -12362,7 +12362,7 @@
       <c r="AG190" s="2"/>
       <c r="AH190" s="2"/>
     </row>
-    <row r="191" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="191" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
       <c r="D191" s="2"/>
@@ -12397,7 +12397,7 @@
       <c r="AG191" s="2"/>
       <c r="AH191" s="2"/>
     </row>
-    <row r="192" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="192" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B192" s="2"/>
       <c r="C192" s="2"/>
       <c r="D192" s="2"/>
@@ -12432,7 +12432,7 @@
       <c r="AG192" s="2"/>
       <c r="AH192" s="2"/>
     </row>
-    <row r="193" spans="2:37" s="125" customFormat="1" ht="12" customHeight="1">
+    <row r="193" spans="2:37" s="124" customFormat="1" ht="12" customHeight="1">
       <c r="B193" s="2"/>
       <c r="C193" s="2"/>
       <c r="D193" s="2"/>
@@ -12467,7 +12467,7 @@
       <c r="AG193" s="2"/>
       <c r="AH193" s="2"/>
     </row>
-    <row r="194" spans="2:37" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="194" spans="2:37" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="B194" s="2"/>
       <c r="C194" s="2"/>
       <c r="D194" s="2"/>
@@ -12502,7 +12502,7 @@
       <c r="AG194" s="2"/>
       <c r="AH194" s="2"/>
     </row>
-    <row r="195" spans="2:37" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="195" spans="2:37" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="B195" s="2"/>
       <c r="C195" s="2"/>
       <c r="D195" s="2"/>
@@ -12537,7 +12537,7 @@
       <c r="AG195" s="2"/>
       <c r="AH195" s="2"/>
     </row>
-    <row r="196" spans="2:37" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="196" spans="2:37" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="B196" s="2"/>
       <c r="C196" s="2"/>
       <c r="D196" s="2"/>
@@ -12572,7 +12572,7 @@
       <c r="AG196" s="2"/>
       <c r="AH196" s="2"/>
     </row>
-    <row r="197" spans="2:37" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="197" spans="2:37" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="B197" s="2"/>
       <c r="C197" s="2"/>
       <c r="D197" s="2"/>
@@ -12607,7 +12607,7 @@
       <c r="AG197" s="2"/>
       <c r="AH197" s="2"/>
     </row>
-    <row r="198" spans="2:37" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="198" spans="2:37" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="B198" s="2"/>
       <c r="C198" s="2"/>
       <c r="D198" s="2"/>
@@ -12642,7 +12642,7 @@
       <c r="AG198" s="2"/>
       <c r="AH198" s="2"/>
     </row>
-    <row r="199" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="199" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B199" s="2"/>
       <c r="C199" s="2"/>
       <c r="D199" s="2"/>
@@ -12677,7 +12677,7 @@
       <c r="AG199" s="2"/>
       <c r="AH199" s="2"/>
     </row>
-    <row r="200" spans="2:37" s="125" customFormat="1" ht="12.75" customHeight="1">
+    <row r="200" spans="2:37" s="124" customFormat="1" ht="12.75" customHeight="1">
       <c r="B200" s="2"/>
       <c r="C200" s="2"/>
       <c r="D200" s="2"/>
@@ -12712,7 +12712,7 @@
       <c r="AG200" s="2"/>
       <c r="AH200" s="2"/>
     </row>
-    <row r="201" spans="2:37" s="125" customFormat="1">
+    <row r="201" spans="2:37" s="124" customFormat="1">
       <c r="B201" s="2"/>
       <c r="C201" s="2"/>
       <c r="D201" s="2"/>
@@ -12750,7 +12750,7 @@
       <c r="AJ201" s="2"/>
       <c r="AK201" s="2"/>
     </row>
-    <row r="202" spans="2:37" s="125" customFormat="1">
+    <row r="202" spans="2:37" s="124" customFormat="1">
       <c r="B202" s="2"/>
       <c r="C202" s="2"/>
       <c r="D202" s="2"/>
@@ -12788,7 +12788,7 @@
       <c r="AJ202" s="2"/>
       <c r="AK202" s="2"/>
     </row>
-    <row r="203" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="203" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B203" s="2"/>
       <c r="C203" s="2"/>
       <c r="D203" s="2"/>
@@ -12826,7 +12826,7 @@
       <c r="AJ203" s="2"/>
       <c r="AK203" s="2"/>
     </row>
-    <row r="204" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="204" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B204" s="2"/>
       <c r="C204" s="2"/>
       <c r="D204" s="2"/>
@@ -12864,7 +12864,7 @@
       <c r="AJ204" s="2"/>
       <c r="AK204" s="2"/>
     </row>
-    <row r="205" spans="2:37" s="125" customFormat="1">
+    <row r="205" spans="2:37" s="124" customFormat="1">
       <c r="B205" s="2"/>
       <c r="C205" s="2"/>
       <c r="D205" s="2"/>
@@ -12902,7 +12902,7 @@
       <c r="AJ205" s="2"/>
       <c r="AK205" s="2"/>
     </row>
-    <row r="206" spans="2:37" s="125" customFormat="1" ht="24">
+    <row r="206" spans="2:37" s="124" customFormat="1" ht="24">
       <c r="B206" s="2"/>
       <c r="C206" s="2"/>
       <c r="D206" s="2"/>
@@ -12936,11 +12936,11 @@
       <c r="AF206" s="2"/>
       <c r="AG206" s="2"/>
       <c r="AH206" s="2"/>
-      <c r="AI206" s="126"/>
-      <c r="AJ206" s="126"/>
-      <c r="AK206" s="126"/>
-    </row>
-    <row r="207" spans="2:37" s="125" customFormat="1">
+      <c r="AI206" s="125"/>
+      <c r="AJ206" s="125"/>
+      <c r="AK206" s="125"/>
+    </row>
+    <row r="207" spans="2:37" s="124" customFormat="1">
       <c r="B207" s="2"/>
       <c r="C207" s="2"/>
       <c r="D207" s="2"/>
@@ -12978,7 +12978,7 @@
       <c r="AJ207" s="2"/>
       <c r="AK207" s="2"/>
     </row>
-    <row r="208" spans="2:37" s="125" customFormat="1" ht="20.25" customHeight="1">
+    <row r="208" spans="2:37" s="124" customFormat="1" ht="20.25" customHeight="1">
       <c r="B208" s="2"/>
       <c r="C208" s="2"/>
       <c r="D208" s="2"/>
@@ -13016,7 +13016,7 @@
       <c r="AJ208" s="2"/>
       <c r="AK208" s="2"/>
     </row>
-    <row r="209" spans="1:59" s="125" customFormat="1">
+    <row r="209" spans="1:59" s="124" customFormat="1">
       <c r="B209" s="2"/>
       <c r="C209" s="2"/>
       <c r="D209" s="2"/>
@@ -13055,7 +13055,7 @@
       <c r="AK209" s="2"/>
     </row>
     <row r="210" spans="1:59" ht="20.25" customHeight="1"/>
-    <row r="215" spans="1:59" s="126" customFormat="1" ht="24">
+    <row r="215" spans="1:59" s="125" customFormat="1" ht="24">
       <c r="B215" s="2"/>
       <c r="C215" s="2"/>
       <c r="D215" s="2"/>
@@ -13156,22 +13156,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="E35:R36"/>
-    <mergeCell ref="B61:U62"/>
-    <mergeCell ref="V26:V27"/>
-    <mergeCell ref="W26:AJ26"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="Z23:AB23"/>
-    <mergeCell ref="AC23:AE23"/>
-    <mergeCell ref="AF23:AH23"/>
-    <mergeCell ref="W24:Y24"/>
-    <mergeCell ref="Z24:AB24"/>
-    <mergeCell ref="AC24:AE24"/>
-    <mergeCell ref="AF24:AH24"/>
     <mergeCell ref="W8:AM8"/>
     <mergeCell ref="C9:H9"/>
     <mergeCell ref="B2:AN2"/>
@@ -13186,6 +13170,22 @@
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="R8:S8"/>
     <mergeCell ref="V8:V9"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="Z23:AB23"/>
+    <mergeCell ref="AC23:AE23"/>
+    <mergeCell ref="AF23:AH23"/>
+    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="Z24:AB24"/>
+    <mergeCell ref="AC24:AE24"/>
+    <mergeCell ref="AF24:AH24"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="E35:R36"/>
+    <mergeCell ref="B61:U62"/>
+    <mergeCell ref="V26:V27"/>
+    <mergeCell ref="W26:AJ26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.55118110236220474" right="0.35433070866141736" top="0.74803149606299213" bottom="0.74803149606299213" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>